<commit_message>
feat: Finalize fishing system and documentation
</commit_message>
<xml_diff>
--- a/Assets/ExcelData/FishData.xlsx
+++ b/Assets/ExcelData/FishData.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="178">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -29,7 +29,10 @@
     <t xml:space="preserve">Price (Gold)</t>
   </si>
   <si>
-    <t xml:space="preserve">Length (cm)</t>
+    <t xml:space="preserve">Min Length (cm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Max Length (cm)</t>
   </si>
   <si>
     <t xml:space="preserve">Description</t>
@@ -41,7 +44,7 @@
     <t xml:space="preserve">악어</t>
   </si>
   <si>
-    <t xml:space="preserve">S</t>
+    <t xml:space="preserve">★★★★★</t>
   </si>
   <si>
     <t xml:space="preserve">늪지의 공포, 거대한 이빨을 가진 지배자입니다.</t>
@@ -62,7 +65,7 @@
     <t xml:space="preserve">큰입배스</t>
   </si>
   <si>
-    <t xml:space="preserve">D</t>
+    <t xml:space="preserve">★</t>
   </si>
   <si>
     <t xml:space="preserve">흔하지만 손맛이 좋은 민물의 강자입니다.</t>
@@ -83,7 +86,7 @@
     <t xml:space="preserve">보우핀</t>
   </si>
   <si>
-    <t xml:space="preserve">C</t>
+    <t xml:space="preserve">★★</t>
   </si>
   <si>
     <t xml:space="preserve">살아있는 화석이라 불리는 튼튼한 물고기입니다.</t>
@@ -95,7 +98,7 @@
     <t xml:space="preserve">황소상어</t>
   </si>
   <si>
-    <t xml:space="preserve">A</t>
+    <t xml:space="preserve">★★★★</t>
   </si>
   <si>
     <t xml:space="preserve">강까지 거슬러 올라오는 아주 위험한 상어입니다.</t>
@@ -170,7 +173,7 @@
     <t xml:space="preserve">가아</t>
   </si>
   <si>
-    <t xml:space="preserve">B</t>
+    <t xml:space="preserve">★★★</t>
   </si>
   <si>
     <t xml:space="preserve">악어 같은 입을 가진 고대의 포식자입니다.</t>
@@ -227,9 +230,6 @@
     <t xml:space="preserve">거머리</t>
   </si>
   <si>
-    <t xml:space="preserve">E</t>
-  </si>
-  <si>
     <t xml:space="preserve">피를 빨아먹는 끈질긴 녀석입니다.</t>
   </si>
   <si>
@@ -519,36 +519,6 @@
   </si>
   <si>
     <t xml:space="preserve">이건 물고기가 아닌 것 같은데... 외계에서 왔을까요?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Min Size (cm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Max Size (cm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">800</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">60</t>
-  </si>
-  <si>
-    <t xml:space="preserve">250</t>
-  </si>
-  <si>
-    <t xml:space="preserve">120</t>
-  </si>
-  <si>
-    <t xml:space="preserve">50</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1000</t>
-  </si>
-  <si>
-    <t xml:space="preserve"/>
   </si>
   <si>
     <t xml:space="preserve">EXP Reward</t>
@@ -640,27 +610,27 @@
         <v>4</v>
       </c>
       <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
         <v>169</v>
-      </c>
-      <c r="G1" t="s">
-        <v>170</v>
-      </c>
-      <c r="H1" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D2">
         <v>0.100000001490116</v>
@@ -672,10 +642,10 @@
         <v>200</v>
       </c>
       <c r="G2">
-        <v>800</v>
+        <v>350</v>
       </c>
       <c r="H2" t="s">
-        <v>180</v>
+        <v>170</v>
       </c>
       <c r="I2">
         <v>5000</v>
@@ -683,13 +653,13 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D3">
         <v>0.0500000007450581</v>
@@ -698,13 +668,13 @@
         <v>9999</v>
       </c>
       <c r="F3">
-        <v>200</v>
+        <v>10</v>
       </c>
       <c r="G3">
-        <v>800</v>
+        <v>25</v>
       </c>
       <c r="H3" t="s">
-        <v>181</v>
+        <v>171</v>
       </c>
       <c r="I3">
         <v>5000</v>
@@ -712,13 +682,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D4">
         <v>8</v>
@@ -727,13 +697,13 @@
         <v>100</v>
       </c>
       <c r="F4">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="G4">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="H4" t="s">
-        <v>182</v>
+        <v>172</v>
       </c>
       <c r="I4">
         <v>20</v>
@@ -741,13 +711,13 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D5">
         <v>10</v>
@@ -756,13 +726,13 @@
         <v>80</v>
       </c>
       <c r="F5">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G5">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="H5" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I5">
         <v>20</v>
@@ -770,13 +740,13 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D6">
         <v>4</v>
@@ -785,13 +755,13 @@
         <v>250</v>
       </c>
       <c r="F6">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="G6">
         <v>60</v>
       </c>
       <c r="H6" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I6">
         <v>80</v>
@@ -799,13 +769,13 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D7">
         <v>0.5</v>
@@ -814,13 +784,13 @@
         <v>3500</v>
       </c>
       <c r="F7">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="G7">
-        <v>250</v>
+        <v>220</v>
       </c>
       <c r="H7" t="s">
-        <v>184</v>
+        <v>174</v>
       </c>
       <c r="I7">
         <v>1000</v>
@@ -828,13 +798,13 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D8">
         <v>5</v>
@@ -843,13 +813,13 @@
         <v>300</v>
       </c>
       <c r="F8">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="G8">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="H8" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I8">
         <v>80</v>
@@ -857,13 +827,13 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C9" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D9">
         <v>7</v>
@@ -872,13 +842,13 @@
         <v>150</v>
       </c>
       <c r="F9">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="G9">
-        <v>25</v>
+        <v>80</v>
       </c>
       <c r="H9" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I9">
         <v>20</v>
@@ -886,13 +856,13 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D10">
         <v>6</v>
@@ -904,10 +874,10 @@
         <v>5</v>
       </c>
       <c r="G10">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="H10" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I10">
         <v>20</v>
@@ -915,13 +885,13 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B11" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D11">
         <v>9</v>
@@ -930,13 +900,13 @@
         <v>90</v>
       </c>
       <c r="F11">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="G11">
         <v>25</v>
       </c>
       <c r="H11" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I11">
         <v>20</v>
@@ -944,13 +914,13 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C12" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D12">
         <v>8.5</v>
@@ -962,10 +932,10 @@
         <v>5</v>
       </c>
       <c r="G12">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="H12" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I12">
         <v>20</v>
@@ -973,13 +943,13 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C13" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D13">
         <v>3.5</v>
@@ -988,13 +958,13 @@
         <v>400</v>
       </c>
       <c r="F13">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="G13">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H13" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I13">
         <v>80</v>
@@ -1002,13 +972,13 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B14" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D14">
         <v>10</v>
@@ -1017,13 +987,13 @@
         <v>50</v>
       </c>
       <c r="F14">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G14">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="H14" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I14">
         <v>20</v>
@@ -1031,13 +1001,13 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B15" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C15" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D15">
         <v>1.5</v>
@@ -1046,13 +1016,13 @@
         <v>1200</v>
       </c>
       <c r="F15">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="G15">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="H15" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I15">
         <v>250</v>
@@ -1060,13 +1030,13 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B16" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C16" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D16">
         <v>0.100000001490116</v>
@@ -1075,13 +1045,13 @@
         <v>7777</v>
       </c>
       <c r="F16">
-        <v>200</v>
+        <v>30</v>
       </c>
       <c r="G16">
-        <v>800</v>
+        <v>50</v>
       </c>
       <c r="H16" t="s">
-        <v>182</v>
+        <v>172</v>
       </c>
       <c r="I16">
         <v>5000</v>
@@ -1089,13 +1059,13 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B17" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C17" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D17">
         <v>5</v>
@@ -1107,10 +1077,10 @@
         <v>5</v>
       </c>
       <c r="G17">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="H17" t="s">
-        <v>185</v>
+        <v>175</v>
       </c>
       <c r="I17">
         <v>20</v>
@@ -1118,13 +1088,13 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B18" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C18" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D18">
         <v>12</v>
@@ -1133,13 +1103,13 @@
         <v>40</v>
       </c>
       <c r="F18">
+        <v>2</v>
+      </c>
+      <c r="G18">
         <v>5</v>
       </c>
-      <c r="G18">
-        <v>25</v>
-      </c>
       <c r="H18" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I18">
         <v>20</v>
@@ -1147,13 +1117,13 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B19" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C19" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D19">
         <v>0.800000011920929</v>
@@ -1162,13 +1132,13 @@
         <v>2500</v>
       </c>
       <c r="F19">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="G19">
-        <v>250</v>
+        <v>120</v>
       </c>
       <c r="H19" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I19">
         <v>1000</v>
@@ -1176,13 +1146,13 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B20" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C20" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D20">
         <v>2</v>
@@ -1191,13 +1161,13 @@
         <v>1500</v>
       </c>
       <c r="F20">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="G20">
-        <v>120</v>
+        <v>65</v>
       </c>
       <c r="H20" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I20">
         <v>250</v>
@@ -1205,13 +1175,13 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B21" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C21" t="s">
-        <v>71</v>
+        <v>17</v>
       </c>
       <c r="D21">
         <v>10</v>
@@ -1220,16 +1190,16 @@
         <v>10</v>
       </c>
       <c r="F21">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="G21">
-        <v>50</v>
+        <v>5</v>
       </c>
       <c r="H21" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I21">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22">
@@ -1240,7 +1210,7 @@
         <v>74</v>
       </c>
       <c r="C22" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D22">
         <v>3</v>
@@ -1249,13 +1219,13 @@
         <v>350</v>
       </c>
       <c r="F22">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G22">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="H22" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I22">
         <v>80</v>
@@ -1269,7 +1239,7 @@
         <v>77</v>
       </c>
       <c r="C23" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D23">
         <v>1.20000004768372</v>
@@ -1278,13 +1248,13 @@
         <v>1800</v>
       </c>
       <c r="F23">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="G23">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="H23" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I23">
         <v>250</v>
@@ -1298,7 +1268,7 @@
         <v>80</v>
       </c>
       <c r="C24" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D24">
         <v>8</v>
@@ -1307,13 +1277,13 @@
         <v>130</v>
       </c>
       <c r="F24">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="G24">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="H24" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I24">
         <v>20</v>
@@ -1327,7 +1297,7 @@
         <v>83</v>
       </c>
       <c r="C25" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D25">
         <v>2.5</v>
@@ -1339,10 +1309,10 @@
         <v>50</v>
       </c>
       <c r="G25">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="H25" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I25">
         <v>250</v>
@@ -1356,7 +1326,7 @@
         <v>86</v>
       </c>
       <c r="C26" t="s">
-        <v>71</v>
+        <v>17</v>
       </c>
       <c r="D26">
         <v>0.200000002980232</v>
@@ -1365,16 +1335,16 @@
         <v>5000</v>
       </c>
       <c r="F26">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="G26">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="H26" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I26">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="27">
@@ -1385,7 +1355,7 @@
         <v>89</v>
       </c>
       <c r="C27" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D27">
         <v>3</v>
@@ -1394,13 +1364,13 @@
         <v>750</v>
       </c>
       <c r="F27">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="G27">
-        <v>120</v>
+        <v>55</v>
       </c>
       <c r="H27" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I27">
         <v>250</v>
@@ -1414,7 +1384,7 @@
         <v>92</v>
       </c>
       <c r="C28" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D28">
         <v>4.5</v>
@@ -1423,13 +1393,13 @@
         <v>550</v>
       </c>
       <c r="F28">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="G28">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="H28" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I28">
         <v>80</v>
@@ -1443,7 +1413,7 @@
         <v>95</v>
       </c>
       <c r="C29" t="s">
-        <v>71</v>
+        <v>17</v>
       </c>
       <c r="D29">
         <v>15</v>
@@ -1452,16 +1422,16 @@
         <v>20</v>
       </c>
       <c r="F29">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="G29">
-        <v>50</v>
+        <v>3</v>
       </c>
       <c r="H29" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I29">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="30">
@@ -1472,7 +1442,7 @@
         <v>98</v>
       </c>
       <c r="C30" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D30">
         <v>0.400000005960464</v>
@@ -1487,7 +1457,7 @@
         <v>250</v>
       </c>
       <c r="H30" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I30">
         <v>1000</v>
@@ -1501,7 +1471,7 @@
         <v>101</v>
       </c>
       <c r="C31" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D31">
         <v>7</v>
@@ -1513,10 +1483,10 @@
         <v>5</v>
       </c>
       <c r="G31">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="H31" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I31">
         <v>20</v>
@@ -1530,7 +1500,7 @@
         <v>104</v>
       </c>
       <c r="C32" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D32">
         <v>2</v>
@@ -1539,13 +1509,13 @@
         <v>1200</v>
       </c>
       <c r="F32">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G32">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="H32" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I32">
         <v>80</v>
@@ -1559,7 +1529,7 @@
         <v>107</v>
       </c>
       <c r="C33" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D33">
         <v>3.79999995231628</v>
@@ -1568,13 +1538,13 @@
         <v>450</v>
       </c>
       <c r="F33">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="G33">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="H33" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I33">
         <v>250</v>
@@ -1588,7 +1558,7 @@
         <v>110</v>
       </c>
       <c r="C34" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D34">
         <v>4</v>
@@ -1597,13 +1567,13 @@
         <v>600</v>
       </c>
       <c r="F34">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="G34">
-        <v>250</v>
+        <v>20</v>
       </c>
       <c r="H34" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I34">
         <v>1000</v>
@@ -1617,7 +1587,7 @@
         <v>113</v>
       </c>
       <c r="C35" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D35">
         <v>7.5</v>
@@ -1626,13 +1596,13 @@
         <v>180</v>
       </c>
       <c r="F35">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="G35">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="H35" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I35">
         <v>20</v>
@@ -1646,7 +1616,7 @@
         <v>116</v>
       </c>
       <c r="C36" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D36">
         <v>5.5</v>
@@ -1658,10 +1628,10 @@
         <v>5</v>
       </c>
       <c r="G36">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="H36" t="s">
-        <v>186</v>
+        <v>176</v>
       </c>
       <c r="I36">
         <v>20</v>
@@ -1675,7 +1645,7 @@
         <v>119</v>
       </c>
       <c r="C37" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D37">
         <v>0.0799999982118607</v>
@@ -1684,13 +1654,13 @@
         <v>12000</v>
       </c>
       <c r="F37">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="G37">
-        <v>800</v>
+        <v>180</v>
       </c>
       <c r="H37" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I37">
         <v>5000</v>
@@ -1704,7 +1674,7 @@
         <v>122</v>
       </c>
       <c r="C38" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D38">
         <v>3.20000004768372</v>
@@ -1713,13 +1683,13 @@
         <v>550</v>
       </c>
       <c r="F38">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="G38">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="H38" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I38">
         <v>80</v>
@@ -1733,7 +1703,7 @@
         <v>125</v>
       </c>
       <c r="C39" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D39">
         <v>2.20000004768372</v>
@@ -1742,13 +1712,13 @@
         <v>1100</v>
       </c>
       <c r="F39">
-        <v>5</v>
+        <v>60</v>
       </c>
       <c r="G39">
-        <v>25</v>
+        <v>110</v>
       </c>
       <c r="H39" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I39">
         <v>20</v>
@@ -1762,7 +1732,7 @@
         <v>128</v>
       </c>
       <c r="C40" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D40">
         <v>8.19999980926514</v>
@@ -1771,13 +1741,13 @@
         <v>220</v>
       </c>
       <c r="F40">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="G40">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="H40" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I40">
         <v>20</v>
@@ -1791,7 +1761,7 @@
         <v>131</v>
       </c>
       <c r="C41" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D41">
         <v>1.79999995231628</v>
@@ -1800,13 +1770,13 @@
         <v>1600</v>
       </c>
       <c r="F41">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="G41">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="H41" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I41">
         <v>250</v>
@@ -1820,7 +1790,7 @@
         <v>134</v>
       </c>
       <c r="C42" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D42">
         <v>11</v>
@@ -1829,13 +1799,13 @@
         <v>70</v>
       </c>
       <c r="F42">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="G42">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="H42" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I42">
         <v>20</v>
@@ -1849,7 +1819,7 @@
         <v>137</v>
       </c>
       <c r="C43" t="s">
-        <v>71</v>
+        <v>17</v>
       </c>
       <c r="D43">
         <v>20</v>
@@ -1858,16 +1828,16 @@
         <v>5</v>
       </c>
       <c r="F43">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="G43">
-        <v>50</v>
+        <v>2</v>
       </c>
       <c r="H43" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I43">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="44">
@@ -1878,7 +1848,7 @@
         <v>140</v>
       </c>
       <c r="C44" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D44">
         <v>2</v>
@@ -1887,13 +1857,13 @@
         <v>1300</v>
       </c>
       <c r="F44">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="G44">
-        <v>120</v>
+        <v>35</v>
       </c>
       <c r="H44" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I44">
         <v>250</v>
@@ -1907,7 +1877,7 @@
         <v>143</v>
       </c>
       <c r="C45" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D45">
         <v>1</v>
@@ -1916,13 +1886,13 @@
         <v>3200</v>
       </c>
       <c r="F45">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="G45">
-        <v>250</v>
+        <v>45</v>
       </c>
       <c r="H45" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I45">
         <v>1000</v>
@@ -1936,7 +1906,7 @@
         <v>146</v>
       </c>
       <c r="C46" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D46">
         <v>0.699999988079071</v>
@@ -1945,13 +1915,13 @@
         <v>5500</v>
       </c>
       <c r="F46">
-        <v>100</v>
+        <v>15</v>
       </c>
       <c r="G46">
-        <v>250</v>
+        <v>30</v>
       </c>
       <c r="H46" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I46">
         <v>1000</v>
@@ -1965,7 +1935,7 @@
         <v>149</v>
       </c>
       <c r="C47" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D47">
         <v>1.5</v>
@@ -1974,13 +1944,13 @@
         <v>2200</v>
       </c>
       <c r="F47">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="G47">
-        <v>120</v>
+        <v>250</v>
       </c>
       <c r="H47" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I47">
         <v>250</v>
@@ -1994,7 +1964,7 @@
         <v>152</v>
       </c>
       <c r="C48" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D48">
         <v>0.0500000007450581</v>
@@ -2003,13 +1973,13 @@
         <v>15000</v>
       </c>
       <c r="F48">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="G48">
-        <v>800</v>
+        <v>300</v>
       </c>
       <c r="H48" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I48">
         <v>5000</v>
@@ -2023,7 +1993,7 @@
         <v>155</v>
       </c>
       <c r="C49" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D49">
         <v>0.150000005960464</v>
@@ -2032,13 +2002,13 @@
         <v>9000</v>
       </c>
       <c r="F49">
-        <v>200</v>
+        <v>60</v>
       </c>
       <c r="G49">
-        <v>800</v>
+        <v>120</v>
       </c>
       <c r="H49" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I49">
         <v>5000</v>
@@ -2052,7 +2022,7 @@
         <v>158</v>
       </c>
       <c r="C50" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D50">
         <v>0.0500000007450581</v>
@@ -2061,13 +2031,13 @@
         <v>25000</v>
       </c>
       <c r="F50">
-        <v>200</v>
+        <v>40</v>
       </c>
       <c r="G50">
-        <v>800</v>
+        <v>100</v>
       </c>
       <c r="H50" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I50">
         <v>5000</v>
@@ -2081,7 +2051,7 @@
         <v>161</v>
       </c>
       <c r="C51" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D51">
         <v>0.0500000007450581</v>
@@ -2090,13 +2060,13 @@
         <v>30000</v>
       </c>
       <c r="F51">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="G51">
-        <v>800</v>
+        <v>400</v>
       </c>
       <c r="H51" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I51">
         <v>5000</v>
@@ -2110,7 +2080,7 @@
         <v>164</v>
       </c>
       <c r="C52" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D52">
         <v>0.0199999995529652</v>
@@ -2119,13 +2089,13 @@
         <v>45000</v>
       </c>
       <c r="F52">
-        <v>200</v>
+        <v>800</v>
       </c>
       <c r="G52">
-        <v>800</v>
+        <v>1600</v>
       </c>
       <c r="H52" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I52">
         <v>5000</v>
@@ -2139,7 +2109,7 @@
         <v>167</v>
       </c>
       <c r="C53" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D53">
         <v>0.00999999977648258</v>
@@ -2148,13 +2118,13 @@
         <v>99999</v>
       </c>
       <c r="F53">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="G53">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="H53" t="s">
-        <v>187</v>
+        <v>177</v>
       </c>
       <c r="I53">
         <v>5000</v>

</xml_diff>

<commit_message>
feat: implement weight-based fishing difficulty and sync to Excel
- Added 'weight' and 'requiredSpam' fields to FishDataSO
- Updated ExcelDataConverter to calculate and store required spam clicks (1-10) in Excel
- Modified FishingPlayer to use requiredSpam value from fish data for mini-game difficulty
- Updated all fish SO assets with newly generated weight and difficulty data
</commit_message>
<xml_diff>
--- a/Assets/ExcelData/FishData.xlsx
+++ b/Assets/ExcelData/FishData.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="180">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -546,6 +546,12 @@
   </si>
   <si>
     <t xml:space="preserve">이건 물고기가 아닙니다! 외계에서 날아온 비행 물체네요.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weight</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Required Spam</t>
   </si>
 </sst>
 </file>
@@ -590,7 +596,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:I53"/>
+  <dimension ref="A1:K53"/>
   <sheetFormatPr defaultColWidth="8.43" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -621,6 +627,12 @@
       <c r="I1" t="s">
         <v>169</v>
       </c>
+      <c r="J1" t="s">
+        <v>178</v>
+      </c>
+      <c r="K1" t="s">
+        <v>179</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
@@ -650,6 +662,12 @@
       <c r="I2">
         <v>5000</v>
       </c>
+      <c r="J2">
+        <v>756.25</v>
+      </c>
+      <c r="K2">
+        <v>10</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
@@ -679,6 +697,12 @@
       <c r="I3">
         <v>5000</v>
       </c>
+      <c r="J3">
+        <v>3.05999994277954</v>
+      </c>
+      <c r="K3">
+        <v>7</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
@@ -708,6 +732,12 @@
       <c r="I4">
         <v>20</v>
       </c>
+      <c r="J4">
+        <v>2.10999989509583</v>
+      </c>
+      <c r="K4">
+        <v>3</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
@@ -737,6 +767,12 @@
       <c r="I5">
         <v>20</v>
       </c>
+      <c r="J5">
+        <v>0.449999988079071</v>
+      </c>
+      <c r="K5">
+        <v>2</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
@@ -766,6 +802,12 @@
       <c r="I6">
         <v>80</v>
       </c>
+      <c r="J6">
+        <v>4.46000003814697</v>
+      </c>
+      <c r="K6">
+        <v>4</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
@@ -795,6 +837,12 @@
       <c r="I7">
         <v>1000</v>
       </c>
+      <c r="J7">
+        <v>144.5</v>
+      </c>
+      <c r="K7">
+        <v>8</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
@@ -824,6 +872,12 @@
       <c r="I8">
         <v>80</v>
       </c>
+      <c r="J8">
+        <v>6.65999984741211</v>
+      </c>
+      <c r="K8">
+        <v>4</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
@@ -853,6 +907,12 @@
       <c r="I9">
         <v>20</v>
       </c>
+      <c r="J9">
+        <v>7.19999980926514</v>
+      </c>
+      <c r="K9">
+        <v>3</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
@@ -882,6 +942,12 @@
       <c r="I10">
         <v>20</v>
       </c>
+      <c r="J10">
+        <v>0.200000002980232</v>
+      </c>
+      <c r="K10">
+        <v>2</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
@@ -911,6 +977,12 @@
       <c r="I11">
         <v>20</v>
       </c>
+      <c r="J11">
+        <v>0.800000011920929</v>
+      </c>
+      <c r="K11">
+        <v>2</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
@@ -940,6 +1012,12 @@
       <c r="I12">
         <v>20</v>
       </c>
+      <c r="J12">
+        <v>0.109999999403954</v>
+      </c>
+      <c r="K12">
+        <v>2</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
@@ -969,6 +1047,12 @@
       <c r="I13">
         <v>80</v>
       </c>
+      <c r="J13">
+        <v>3.08999991416931</v>
+      </c>
+      <c r="K13">
+        <v>4</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
@@ -998,6 +1082,12 @@
       <c r="I14">
         <v>20</v>
       </c>
+      <c r="J14">
+        <v>0.0599999986588955</v>
+      </c>
+      <c r="K14">
+        <v>2</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
@@ -1027,6 +1117,12 @@
       <c r="I15">
         <v>250</v>
       </c>
+      <c r="J15">
+        <v>39.6800003051758</v>
+      </c>
+      <c r="K15">
+        <v>6</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
@@ -1056,6 +1152,12 @@
       <c r="I16">
         <v>5000</v>
       </c>
+      <c r="J16">
+        <v>16</v>
+      </c>
+      <c r="K16">
+        <v>8</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
@@ -1085,6 +1187,12 @@
       <c r="I17">
         <v>20</v>
       </c>
+      <c r="J17">
+        <v>0.200000002980232</v>
+      </c>
+      <c r="K17">
+        <v>2</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
@@ -1114,6 +1222,12 @@
       <c r="I18">
         <v>20</v>
       </c>
+      <c r="J18">
+        <v>0.0199999995529652</v>
+      </c>
+      <c r="K18">
+        <v>2</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
@@ -1143,6 +1257,12 @@
       <c r="I19">
         <v>1000</v>
       </c>
+      <c r="J19">
+        <v>50</v>
+      </c>
+      <c r="K19">
+        <v>8</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
@@ -1172,6 +1292,12 @@
       <c r="I20">
         <v>250</v>
       </c>
+      <c r="J20">
+        <v>6.76999998092651</v>
+      </c>
+      <c r="K20">
+        <v>5</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
@@ -1201,6 +1327,12 @@
       <c r="I21">
         <v>20</v>
       </c>
+      <c r="J21">
+        <v>0.0199999995529652</v>
+      </c>
+      <c r="K21">
+        <v>2</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
@@ -1230,6 +1362,12 @@
       <c r="I22">
         <v>80</v>
       </c>
+      <c r="J22">
+        <v>1.11000001430511</v>
+      </c>
+      <c r="K22">
+        <v>3</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
@@ -1259,6 +1397,12 @@
       <c r="I23">
         <v>250</v>
       </c>
+      <c r="J23">
+        <v>30</v>
+      </c>
+      <c r="K23">
+        <v>6</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
@@ -1288,6 +1432,12 @@
       <c r="I24">
         <v>20</v>
       </c>
+      <c r="J24">
+        <v>1.25</v>
+      </c>
+      <c r="K24">
+        <v>3</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
@@ -1317,6 +1467,12 @@
       <c r="I25">
         <v>250</v>
       </c>
+      <c r="J25">
+        <v>16.8799991607666</v>
+      </c>
+      <c r="K25">
+        <v>6</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
@@ -1346,6 +1502,12 @@
       <c r="I26">
         <v>20</v>
       </c>
+      <c r="J26">
+        <v>0.00999999977648258</v>
+      </c>
+      <c r="K26">
+        <v>2</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
@@ -1375,6 +1537,12 @@
       <c r="I27">
         <v>250</v>
       </c>
+      <c r="J27">
+        <v>5.42000007629395</v>
+      </c>
+      <c r="K27">
+        <v>5</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
@@ -1404,6 +1572,12 @@
       <c r="I28">
         <v>80</v>
       </c>
+      <c r="J28">
+        <v>7.92000007629395</v>
+      </c>
+      <c r="K28">
+        <v>4</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
@@ -1433,6 +1607,12 @@
       <c r="I29">
         <v>20</v>
       </c>
+      <c r="J29">
+        <v>0.00999999977648258</v>
+      </c>
+      <c r="K29">
+        <v>2</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
@@ -1462,6 +1642,12 @@
       <c r="I30">
         <v>1000</v>
       </c>
+      <c r="J30">
+        <v>153.119995117188</v>
+      </c>
+      <c r="K30">
+        <v>8</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
@@ -1491,6 +1677,12 @@
       <c r="I31">
         <v>20</v>
       </c>
+      <c r="J31">
+        <v>0.140000000596046</v>
+      </c>
+      <c r="K31">
+        <v>2</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
@@ -1520,6 +1712,12 @@
       <c r="I32">
         <v>80</v>
       </c>
+      <c r="J32">
+        <v>1.6599999666214</v>
+      </c>
+      <c r="K32">
+        <v>4</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
@@ -1549,6 +1747,12 @@
       <c r="I33">
         <v>250</v>
       </c>
+      <c r="J33">
+        <v>6.07999992370605</v>
+      </c>
+      <c r="K33">
+        <v>5</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
@@ -1578,6 +1782,12 @@
       <c r="I34">
         <v>1000</v>
       </c>
+      <c r="J34">
+        <v>1.12000000476837</v>
+      </c>
+      <c r="K34">
+        <v>5</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
@@ -1607,6 +1817,12 @@
       <c r="I35">
         <v>20</v>
       </c>
+      <c r="J35">
+        <v>2.80999994277954</v>
+      </c>
+      <c r="K35">
+        <v>3</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
@@ -1636,6 +1852,12 @@
       <c r="I36">
         <v>20</v>
       </c>
+      <c r="J36">
+        <v>0.109999999403954</v>
+      </c>
+      <c r="K36">
+        <v>2</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
@@ -1665,6 +1887,12 @@
       <c r="I37">
         <v>5000</v>
       </c>
+      <c r="J37">
+        <v>196</v>
+      </c>
+      <c r="K37">
+        <v>9</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
@@ -1694,6 +1922,12 @@
       <c r="I38">
         <v>80</v>
       </c>
+      <c r="J38">
+        <v>12.3800001144409</v>
+      </c>
+      <c r="K38">
+        <v>5</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
@@ -1723,6 +1957,12 @@
       <c r="I39">
         <v>20</v>
       </c>
+      <c r="J39">
+        <v>14.4499998092651</v>
+      </c>
+      <c r="K39">
+        <v>4</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="s">
@@ -1752,6 +1992,12 @@
       <c r="I40">
         <v>20</v>
       </c>
+      <c r="J40">
+        <v>1.79999995231628</v>
+      </c>
+      <c r="K40">
+        <v>3</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="s">
@@ -1781,6 +2027,12 @@
       <c r="I41">
         <v>250</v>
       </c>
+      <c r="J41">
+        <v>39.6800003051758</v>
+      </c>
+      <c r="K41">
+        <v>6</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
@@ -1810,6 +2062,12 @@
       <c r="I42">
         <v>20</v>
       </c>
+      <c r="J42">
+        <v>1.00999999046326</v>
+      </c>
+      <c r="K42">
+        <v>2</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
@@ -1839,6 +2097,12 @@
       <c r="I43">
         <v>20</v>
       </c>
+      <c r="J43">
+        <v>0</v>
+      </c>
+      <c r="K43">
+        <v>2</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="s">
@@ -1868,6 +2132,12 @@
       <c r="I44">
         <v>250</v>
       </c>
+      <c r="J44">
+        <v>1.87999999523163</v>
+      </c>
+      <c r="K44">
+        <v>5</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="s">
@@ -1897,6 +2167,12 @@
       <c r="I45">
         <v>1000</v>
       </c>
+      <c r="J45">
+        <v>5.28000020980835</v>
+      </c>
+      <c r="K45">
+        <v>6</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="s">
@@ -1926,6 +2202,12 @@
       <c r="I46">
         <v>1000</v>
       </c>
+      <c r="J46">
+        <v>2.52999997138977</v>
+      </c>
+      <c r="K46">
+        <v>6</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="s">
@@ -1955,6 +2237,12 @@
       <c r="I47">
         <v>250</v>
       </c>
+      <c r="J47">
+        <v>91.879997253418</v>
+      </c>
+      <c r="K47">
+        <v>7</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="s">
@@ -1984,6 +2272,12 @@
       <c r="I48">
         <v>5000</v>
       </c>
+      <c r="J48">
+        <v>506.25</v>
+      </c>
+      <c r="K48">
+        <v>10</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="s">
@@ -2013,6 +2307,12 @@
       <c r="I49">
         <v>5000</v>
       </c>
+      <c r="J49">
+        <v>81</v>
+      </c>
+      <c r="K49">
+        <v>9</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="s">
@@ -2042,6 +2342,12 @@
       <c r="I50">
         <v>5000</v>
       </c>
+      <c r="J50">
+        <v>49</v>
+      </c>
+      <c r="K50">
+        <v>9</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="s">
@@ -2071,6 +2377,12 @@
       <c r="I51">
         <v>5000</v>
       </c>
+      <c r="J51">
+        <v>756.25</v>
+      </c>
+      <c r="K51">
+        <v>10</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="s">
@@ -2100,6 +2412,12 @@
       <c r="I52">
         <v>5000</v>
       </c>
+      <c r="J52">
+        <v>14400</v>
+      </c>
+      <c r="K52">
+        <v>10</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="s">
@@ -2128,6 +2446,12 @@
       </c>
       <c r="I53">
         <v>5000</v>
+      </c>
+      <c r="J53">
+        <v>900</v>
+      </c>
+      <c r="K53">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: implement shop system with rod/bait data, buy/equip mechanics, and ShopUI
- Add RodDataSO/BaitDataSO data models with Excel converter support
- Extend IDataService/IUserService with rod/bait queries and buy/equip APIs
- Implement UserStorageService.BuyItem/EquipRod/EquipBait/Unequip
- Add FishingPlayer SyncVar for equipped items with Command/Rpc network flow
- Create ShopUI with category tabs (rods/baits/sell) and detail panel
- Add ShopInventoryPanel with sell-all confirm dialog linked to inventory
- Include UI_SETUP_GUIDE.md for prefab setup (steps 3-7 need Unity Editor)
</commit_message>
<xml_diff>
--- a/Assets/ExcelData/FishData.xlsx
+++ b/Assets/ExcelData/FishData.xlsx
@@ -1,570 +1,559 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <workbookPr autoCompressPictures="1"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <workbookPr defaultThemeVersion="166925"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Unity\MultiplayFishingGame\Assets\ExcelData\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_CF4A63481BB9D411202F87246475D13240D807F7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView tabRatio="600"/>
+    <workbookView xWindow="3075" yWindow="3075" windowWidth="21600" windowHeight="11385" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="FishList" sheetId="1" r:id="rId3"/>
+    <sheet name="FishList" sheetId="1" r:id="rId1"/>
+    <sheet name="Rods" sheetId="2" r:id="rId2"/>
+    <sheet name="Baits" sheetId="3" r:id="rId3"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="180">
-  <si>
-    <t xml:space="preserve">ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rank</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chance (%)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Price (Gold)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Min Length (cm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Max Length (cm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Description</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_alligator</t>
-  </si>
-  <si>
-    <t xml:space="preserve">악어</t>
-  </si>
-  <si>
-    <t xml:space="preserve">★★★★★</t>
-  </si>
-  <si>
-    <t xml:space="preserve">늪지의 공포, 거대한 이빨을 가진 지배자입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_axolotl</t>
-  </si>
-  <si>
-    <t xml:space="preserve">아홀로틀</t>
-  </si>
-  <si>
-    <t xml:space="preserve">웃고 있는 비밀의 수호자, 핑크빛 신비입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_bass</t>
-  </si>
-  <si>
-    <t xml:space="preserve">큰입배스</t>
-  </si>
-  <si>
-    <t xml:space="preserve">★</t>
-  </si>
-  <si>
-    <t xml:space="preserve">흔하지만 손맛이 좋은 민물의 강자입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_bluegill</t>
-  </si>
-  <si>
-    <t xml:space="preserve">블루길</t>
-  </si>
-  <si>
-    <t xml:space="preserve">파란색 아가미를 가진 작고 흔한 물고기입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_bowfin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">보우핀</t>
-  </si>
-  <si>
-    <t xml:space="preserve">★★</t>
-  </si>
-  <si>
-    <t xml:space="preserve">살아있는 화석이라 불리는 튼튼한 물고기입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_bullshark</t>
-  </si>
-  <si>
-    <t xml:space="preserve">황소상어</t>
-  </si>
-  <si>
-    <t xml:space="preserve">★★★★</t>
-  </si>
-  <si>
-    <t xml:space="preserve">강까지 거슬러 올라오는 아주 위험한 상어입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_carp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">잉어</t>
-  </si>
-  <si>
-    <t xml:space="preserve">강인한 생명력의 상징, 영리한 민물고기입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_catfish</t>
-  </si>
-  <si>
-    <t xml:space="preserve">메기</t>
-  </si>
-  <si>
-    <t xml:space="preserve">긴 수염을 가진 바닥의 청소부입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_crab</t>
-  </si>
-  <si>
-    <t xml:space="preserve">게</t>
-  </si>
-  <si>
-    <t xml:space="preserve">옆으로 걷는 집게손의 달인입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_crappie</t>
-  </si>
-  <si>
-    <t xml:space="preserve">크래피</t>
-  </si>
-  <si>
-    <t xml:space="preserve">작지만 군집 생활을 하는 흔한 민물고기입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_crayfish</t>
-  </si>
-  <si>
-    <t xml:space="preserve">가재</t>
-  </si>
-  <si>
-    <t xml:space="preserve">바위 틈에 숨어 사는 집게벌레입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_drum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">민어</t>
-  </si>
-  <si>
-    <t xml:space="preserve">소리를 내어 대화하는 신기한 물고기입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_frog</t>
-  </si>
-  <si>
-    <t xml:space="preserve">개구리</t>
-  </si>
-  <si>
-    <t xml:space="preserve">폴짝폴짝 뛰어다니는 귀여운 양서류입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_gar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">가아</t>
-  </si>
-  <si>
-    <t xml:space="preserve">★★★</t>
-  </si>
-  <si>
-    <t xml:space="preserve">악어 같은 입을 가진 고대의 포식자입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_bass_golden</t>
-  </si>
-  <si>
-    <t xml:space="preserve">골든 배스</t>
-  </si>
-  <si>
-    <t xml:space="preserve">행운을 상징하는 황금빛 배스입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_goldfish</t>
-  </si>
-  <si>
-    <t xml:space="preserve">금붕어</t>
-  </si>
-  <si>
-    <t xml:space="preserve">연못에서 탈출한 듯한 예쁜 물고기입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_guppy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">구피</t>
-  </si>
-  <si>
-    <t xml:space="preserve">작고 화려한 지느러미를 가진 물고기입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_salmon_king</t>
-  </si>
-  <si>
-    <t xml:space="preserve">왕연어</t>
-  </si>
-  <si>
-    <t xml:space="preserve">연어 중의 왕, 거대한 크기를 자랑합니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_koi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">비단잉어</t>
-  </si>
-  <si>
-    <t xml:space="preserve">아름다운 무늬를 가진 정원의 보석입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_leech</t>
-  </si>
-  <si>
-    <t xml:space="preserve">거머리</t>
-  </si>
-  <si>
-    <t xml:space="preserve">피를 빨아먹는 끈질긴 녀석입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_mooneye</t>
-  </si>
-  <si>
-    <t xml:space="preserve">문아이</t>
-  </si>
-  <si>
-    <t xml:space="preserve">달처럼 큰 눈을 가진 은색 물고기입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_muskellunge</t>
-  </si>
-  <si>
-    <t xml:space="preserve">머스키</t>
-  </si>
-  <si>
-    <t xml:space="preserve">민물의 늑대라 불리는 거대한 포식자입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_perch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">퍼치</t>
-  </si>
-  <si>
-    <t xml:space="preserve">줄무늬가 특징인 대중적인 민물고기입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_pike</t>
-  </si>
-  <si>
-    <t xml:space="preserve">강꼬치고기</t>
-  </si>
-  <si>
-    <t xml:space="preserve">화살처럼 빠른 공격력을 가진 물고기입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_pupfish</t>
-  </si>
-  <si>
-    <t xml:space="preserve">펍피쉬</t>
-  </si>
-  <si>
-    <t xml:space="preserve">사막의 오아시스에 사는 아주 희귀한 작은 물고기입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_trout_rainbow</t>
-  </si>
-  <si>
-    <t xml:space="preserve">무지개송어</t>
-  </si>
-  <si>
-    <t xml:space="preserve">옆면에 아름다운 무지개색 띠가 있습니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_salmon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">연어</t>
-  </si>
-  <si>
-    <t xml:space="preserve">고향을 찾아 돌아오는 맛있는 물고기입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_snail</t>
-  </si>
-  <si>
-    <t xml:space="preserve">달팽이</t>
-  </si>
-  <si>
-    <t xml:space="preserve">느릿느릿 기어다니는 껍질집 주인입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_sturgeon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">철갑상어</t>
-  </si>
-  <si>
-    <t xml:space="preserve">귀한 캐비어를 품고 있는 커다란 물고기입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_toad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">두꺼비</t>
-  </si>
-  <si>
-    <t xml:space="preserve">울퉁불퉁한 피부를 가진 듬직한 양서류입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_turtle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">거북이</t>
-  </si>
-  <si>
-    <t xml:space="preserve">오래 사는 지혜의 상징, 딱딱한 등껍질을 가졌습니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_walleye</t>
-  </si>
-  <si>
-    <t xml:space="preserve">월아이</t>
-  </si>
-  <si>
-    <t xml:space="preserve">밤눈이 밝은 빛나는 눈의 물고기입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_angelfish</t>
-  </si>
-  <si>
-    <t xml:space="preserve">엔젤피쉬</t>
-  </si>
-  <si>
-    <t xml:space="preserve">천사처럼 우아한 지느러미를 가졌습니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_bluefish</t>
-  </si>
-  <si>
-    <t xml:space="preserve">블루피쉬</t>
-  </si>
-  <si>
-    <t xml:space="preserve">성질이 사나운 바다의 파이터입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_clownfish</t>
-  </si>
-  <si>
-    <t xml:space="preserve">흰동가리</t>
-  </si>
-  <si>
-    <t xml:space="preserve">말미잘 속에 숨어 사는 귀여운 니모입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_coelacanth</t>
-  </si>
-  <si>
-    <t xml:space="preserve">실러캔스</t>
-  </si>
-  <si>
-    <t xml:space="preserve">수억 년 전부터 살아온 바다의 살아있는 화석입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_dogfish</t>
-  </si>
-  <si>
-    <t xml:space="preserve">돔발상어</t>
-  </si>
-  <si>
-    <t xml:space="preserve">개처럼 무리를 지어 다니는 작은 상어입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_eel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">장어</t>
-  </si>
-  <si>
-    <t xml:space="preserve">미끌미끌하고 힘이 넘치는 스테미나의 왕입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_flounder</t>
-  </si>
-  <si>
-    <t xml:space="preserve">가자미</t>
-  </si>
-  <si>
-    <t xml:space="preserve">바닥에 딱 붙어 사는 위장의 달인입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_grouper</t>
-  </si>
-  <si>
-    <t xml:space="preserve">그루퍼</t>
-  </si>
-  <si>
-    <t xml:space="preserve">거대한 입으로 무엇이든 삼키는 바다의 대식가입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_herring</t>
-  </si>
-  <si>
-    <t xml:space="preserve">청어</t>
-  </si>
-  <si>
-    <t xml:space="preserve">떼 지어 다니는 은빛 바다의 보석입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_krill</t>
-  </si>
-  <si>
-    <t xml:space="preserve">크릴</t>
-  </si>
-  <si>
-    <t xml:space="preserve">고래들의 훌륭한 식사이자 바다의 기초입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_lionfish</t>
-  </si>
-  <si>
-    <t xml:space="preserve">쏠배감펭</t>
-  </si>
-  <si>
-    <t xml:space="preserve">화려한 가시 속에 독을 품은 아름다운 물고기입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_lobster</t>
-  </si>
-  <si>
-    <t xml:space="preserve">바닷가재</t>
-  </si>
-  <si>
-    <t xml:space="preserve">고급스러운 맛과 강력한 집게를 가졌습니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_manowar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">만오워</t>
-  </si>
-  <si>
-    <t xml:space="preserve">푸른 바다의 위험한 독침 풍선입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_mantaray</t>
-  </si>
-  <si>
-    <t xml:space="preserve">가오리</t>
-  </si>
-  <si>
-    <t xml:space="preserve">바다를 나는 듯이 헤엄치는 거대한 날개입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_mantaray_golden</t>
-  </si>
-  <si>
-    <t xml:space="preserve">황금 가오리</t>
-  </si>
-  <si>
-    <t xml:space="preserve">바다의 보물, 찬란한 황금빛을 내뿜습니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_seaturtle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">바다거북</t>
-  </si>
-  <si>
-    <t xml:space="preserve">대양을 횡단하는 경이로운 여행자입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_anomalocaris</t>
-  </si>
-  <si>
-    <t xml:space="preserve">아노말로카리스</t>
-  </si>
-  <si>
-    <t xml:space="preserve">고대 캄브리아기 바다의 정점 포식자입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_helicoprion</t>
-  </si>
-  <si>
-    <t xml:space="preserve">헬리코프리온</t>
-  </si>
-  <si>
-    <t xml:space="preserve">나선형 이빨을 가진 기괴한 고대 상어입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_leedsichthys</t>
-  </si>
-  <si>
-    <t xml:space="preserve">리드시크티스</t>
-  </si>
-  <si>
-    <t xml:space="preserve">역사상 가장 컸던 거대 물고기입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fish_ufo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UFO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">이건 물고기가 아닌 것 같은데... 외계에서 왔을까요?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EXP Reward</t>
-  </si>
-  <si>
-    <t xml:space="preserve">강의 지배자. 날카로운 이빨을 조심하세요.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">웃는 얼굴의 귀여운 도롱뇽. 보고만 있어도 기분이 좋아집니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">입이 정말 커서 무엇이든 집어삼키는 탐욕스러운 물고기입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">평범하지만 특별한 당신만의 물고기입니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">바다의 최상위 포식자. 잡았다는 것 자체가 기적입니다!</t>
-  </si>
-  <si>
-    <t xml:space="preserve">어항에서 탈출한 걸까요? 반짝이는 비늘이 아름답습니다.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">산호초 사이를 헤엄치는 귀여운 물고기. 영화 속 주인공 같아요.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">이건 물고기가 아닙니다! 외계에서 날아온 비행 물체네요.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weight</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Required Spam</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="171">
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Rank</t>
+  </si>
+  <si>
+    <t>Chance (%)</t>
+  </si>
+  <si>
+    <t>Price (Gold)</t>
+  </si>
+  <si>
+    <t>Min Length (cm)</t>
+  </si>
+  <si>
+    <t>Max Length (cm)</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>fish_alligator</t>
+  </si>
+  <si>
+    <t>악어</t>
+  </si>
+  <si>
+    <t>★★★★★</t>
+  </si>
+  <si>
+    <t>fish_axolotl</t>
+  </si>
+  <si>
+    <t>아홀로틀</t>
+  </si>
+  <si>
+    <t>fish_bass</t>
+  </si>
+  <si>
+    <t>큰입배스</t>
+  </si>
+  <si>
+    <t>★</t>
+  </si>
+  <si>
+    <t>fish_bluegill</t>
+  </si>
+  <si>
+    <t>블루길</t>
+  </si>
+  <si>
+    <t>fish_bowfin</t>
+  </si>
+  <si>
+    <t>보우핀</t>
+  </si>
+  <si>
+    <t>★★</t>
+  </si>
+  <si>
+    <t>fish_bullshark</t>
+  </si>
+  <si>
+    <t>황소상어</t>
+  </si>
+  <si>
+    <t>★★★★</t>
+  </si>
+  <si>
+    <t>fish_carp</t>
+  </si>
+  <si>
+    <t>잉어</t>
+  </si>
+  <si>
+    <t>fish_catfish</t>
+  </si>
+  <si>
+    <t>메기</t>
+  </si>
+  <si>
+    <t>fish_crab</t>
+  </si>
+  <si>
+    <t>게</t>
+  </si>
+  <si>
+    <t>fish_crappie</t>
+  </si>
+  <si>
+    <t>크래피</t>
+  </si>
+  <si>
+    <t>fish_crayfish</t>
+  </si>
+  <si>
+    <t>가재</t>
+  </si>
+  <si>
+    <t>fish_drum</t>
+  </si>
+  <si>
+    <t>민어</t>
+  </si>
+  <si>
+    <t>fish_frog</t>
+  </si>
+  <si>
+    <t>개구리</t>
+  </si>
+  <si>
+    <t>fish_gar</t>
+  </si>
+  <si>
+    <t>가아</t>
+  </si>
+  <si>
+    <t>★★★</t>
+  </si>
+  <si>
+    <t>fish_bass_golden</t>
+  </si>
+  <si>
+    <t>골든 배스</t>
+  </si>
+  <si>
+    <t>fish_goldfish</t>
+  </si>
+  <si>
+    <t>금붕어</t>
+  </si>
+  <si>
+    <t>fish_guppy</t>
+  </si>
+  <si>
+    <t>구피</t>
+  </si>
+  <si>
+    <t>fish_salmon_king</t>
+  </si>
+  <si>
+    <t>왕연어</t>
+  </si>
+  <si>
+    <t>fish_koi</t>
+  </si>
+  <si>
+    <t>비단잉어</t>
+  </si>
+  <si>
+    <t>fish_leech</t>
+  </si>
+  <si>
+    <t>거머리</t>
+  </si>
+  <si>
+    <t>fish_mooneye</t>
+  </si>
+  <si>
+    <t>문아이</t>
+  </si>
+  <si>
+    <t>fish_muskellunge</t>
+  </si>
+  <si>
+    <t>머스키</t>
+  </si>
+  <si>
+    <t>fish_perch</t>
+  </si>
+  <si>
+    <t>퍼치</t>
+  </si>
+  <si>
+    <t>fish_pike</t>
+  </si>
+  <si>
+    <t>강꼬치고기</t>
+  </si>
+  <si>
+    <t>fish_pupfish</t>
+  </si>
+  <si>
+    <t>펍피쉬</t>
+  </si>
+  <si>
+    <t>fish_trout_rainbow</t>
+  </si>
+  <si>
+    <t>무지개송어</t>
+  </si>
+  <si>
+    <t>fish_salmon</t>
+  </si>
+  <si>
+    <t>연어</t>
+  </si>
+  <si>
+    <t>fish_snail</t>
+  </si>
+  <si>
+    <t>달팽이</t>
+  </si>
+  <si>
+    <t>fish_sturgeon</t>
+  </si>
+  <si>
+    <t>철갑상어</t>
+  </si>
+  <si>
+    <t>fish_toad</t>
+  </si>
+  <si>
+    <t>두꺼비</t>
+  </si>
+  <si>
+    <t>fish_turtle</t>
+  </si>
+  <si>
+    <t>거북이</t>
+  </si>
+  <si>
+    <t>fish_walleye</t>
+  </si>
+  <si>
+    <t>월아이</t>
+  </si>
+  <si>
+    <t>fish_angelfish</t>
+  </si>
+  <si>
+    <t>엔젤피쉬</t>
+  </si>
+  <si>
+    <t>fish_bluefish</t>
+  </si>
+  <si>
+    <t>블루피쉬</t>
+  </si>
+  <si>
+    <t>fish_clownfish</t>
+  </si>
+  <si>
+    <t>흰동가리</t>
+  </si>
+  <si>
+    <t>fish_coelacanth</t>
+  </si>
+  <si>
+    <t>실러캔스</t>
+  </si>
+  <si>
+    <t>fish_dogfish</t>
+  </si>
+  <si>
+    <t>돔발상어</t>
+  </si>
+  <si>
+    <t>fish_eel</t>
+  </si>
+  <si>
+    <t>장어</t>
+  </si>
+  <si>
+    <t>fish_flounder</t>
+  </si>
+  <si>
+    <t>가자미</t>
+  </si>
+  <si>
+    <t>fish_grouper</t>
+  </si>
+  <si>
+    <t>그루퍼</t>
+  </si>
+  <si>
+    <t>fish_herring</t>
+  </si>
+  <si>
+    <t>청어</t>
+  </si>
+  <si>
+    <t>fish_krill</t>
+  </si>
+  <si>
+    <t>크릴</t>
+  </si>
+  <si>
+    <t>fish_lionfish</t>
+  </si>
+  <si>
+    <t>쏠배감펭</t>
+  </si>
+  <si>
+    <t>fish_lobster</t>
+  </si>
+  <si>
+    <t>바닷가재</t>
+  </si>
+  <si>
+    <t>fish_manowar</t>
+  </si>
+  <si>
+    <t>만오워</t>
+  </si>
+  <si>
+    <t>fish_mantaray</t>
+  </si>
+  <si>
+    <t>가오리</t>
+  </si>
+  <si>
+    <t>fish_mantaray_golden</t>
+  </si>
+  <si>
+    <t>황금 가오리</t>
+  </si>
+  <si>
+    <t>fish_seaturtle</t>
+  </si>
+  <si>
+    <t>바다거북</t>
+  </si>
+  <si>
+    <t>fish_anomalocaris</t>
+  </si>
+  <si>
+    <t>아노말로카리스</t>
+  </si>
+  <si>
+    <t>fish_helicoprion</t>
+  </si>
+  <si>
+    <t>헬리코프리온</t>
+  </si>
+  <si>
+    <t>fish_leedsichthys</t>
+  </si>
+  <si>
+    <t>리드시크티스</t>
+  </si>
+  <si>
+    <t>fish_ufo</t>
+  </si>
+  <si>
+    <t>UFO</t>
+  </si>
+  <si>
+    <t>EXP Reward</t>
+  </si>
+  <si>
+    <t>강의 지배자. 날카로운 이빨을 조심하세요.</t>
+  </si>
+  <si>
+    <t>웃는 얼굴의 귀여운 도롱뇽. 보고만 있어도 기분이 좋아집니다.</t>
+  </si>
+  <si>
+    <t>입이 정말 커서 무엇이든 집어삼키는 탐욕스러운 물고기입니다.</t>
+  </si>
+  <si>
+    <t>평범하지만 특별한 당신만의 물고기입니다.</t>
+  </si>
+  <si>
+    <t>바다의 최상위 포식자. 잡았다는 것 자체가 기적입니다!</t>
+  </si>
+  <si>
+    <t>어항에서 탈출한 걸까요? 반짝이는 비늘이 아름답습니다.</t>
+  </si>
+  <si>
+    <t>산호초 사이를 헤엄치는 귀여운 물고기. 영화 속 주인공 같아요.</t>
+  </si>
+  <si>
+    <t>이건 물고기가 아닙니다! 외계에서 날아온 비행 물체네요.</t>
+  </si>
+  <si>
+    <t>Weight</t>
+  </si>
+  <si>
+    <t>Required Spam</t>
+  </si>
+  <si>
+    <t>Price</t>
+  </si>
+  <si>
+    <t>CastDistanceBonus</t>
+  </si>
+  <si>
+    <t>CatchChanceBonus</t>
+  </si>
+  <si>
+    <t>Durability</t>
+  </si>
+  <si>
+    <t>rod_basic</t>
+  </si>
+  <si>
+    <t>기본 낚싯대</t>
+  </si>
+  <si>
+    <t>누구나 사용할 수 있는 기본 낚싯대입니다.</t>
+  </si>
+  <si>
+    <t>rod_carbon</t>
+  </si>
+  <si>
+    <t>카본 낚싯대</t>
+  </si>
+  <si>
+    <t>가볍고 튼튼한 카본 소재의 낚싯대입니다.</t>
+  </si>
+  <si>
+    <t>rod_fiberglass</t>
+  </si>
+  <si>
+    <t>유리섬유 낚싯대</t>
+  </si>
+  <si>
+    <t>유리섬유 소재로 제작된 중급 낚싯대입니다.</t>
+  </si>
+  <si>
+    <t>rod_titanium</t>
+  </si>
+  <si>
+    <t>티타늄 낚싯대</t>
+  </si>
+  <si>
+    <t>초경량 티타늄 합금으로 제작된 고급 낚싯대입니다.</t>
+  </si>
+  <si>
+    <t>rod_legendary</t>
+  </si>
+  <si>
+    <t>전설의 낚싯대</t>
+  </si>
+  <si>
+    <t>전설 속에만 존재한다는 궁극의 낚싯대입니다.</t>
+  </si>
+  <si>
+    <t>AttractionFishType</t>
+  </si>
+  <si>
+    <t>bait_basic</t>
+  </si>
+  <si>
+    <t>기본 미끼</t>
+  </si>
+  <si>
+    <t>all</t>
+  </si>
+  <si>
+    <t>아무 물고기나 잡을 수 있는 기본 미끼입니다.</t>
+  </si>
+  <si>
+    <t>bait_worm</t>
+  </si>
+  <si>
+    <t>지렁이</t>
+  </si>
+  <si>
+    <t>freshwater</t>
+  </si>
+  <si>
+    <t>민물고기에게 특히 효과적인 지렁이 미끼입니다.</t>
+  </si>
+  <si>
+    <t>bait_shrimp</t>
+  </si>
+  <si>
+    <t>새우</t>
+  </si>
+  <si>
+    <t>saltwater</t>
+  </si>
+  <si>
+    <t>바닷물고기에게 특히 효과적인 새우 미끼입니다.</t>
+  </si>
+  <si>
+    <t>bait_lure</t>
+  </si>
+  <si>
+    <t>루어</t>
+  </si>
+  <si>
+    <t>모든 물고기에게 효과가 좋은 인공 미끼입니다.</t>
+  </si>
+  <si>
+    <t>bait_golden</t>
+  </si>
+  <si>
+    <t>황금 미끼</t>
+  </si>
+  <si>
+    <t>rare</t>
+  </si>
+  <si>
+    <t>희귀 물고기를 유인하는 황금빛 미끼입니다.</t>
+  </si>
+  <si>
+    <t>bait_ancient</t>
+  </si>
+  <si>
+    <t>고대의 미끼</t>
+  </si>
+  <si>
+    <t>legendary</t>
+  </si>
+  <si>
+    <t>고대 바다 생물을 끌어당기는 신비로운 미끼입니다.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -573,7 +562,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="darkGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
@@ -586,20 +575,332 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="표준" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 테마">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="44546A"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="E7E6E6"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4472C4"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="ED7D31"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="A5A5A5"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="FFC000"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="5B9BD5"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="70AD47"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0563C1"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="954F72"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+    </a:ext>
+  </a:extLst>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K53"/>
-  <sheetFormatPr defaultColWidth="8.43" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.375" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -625,16 +926,16 @@
         <v>7</v>
       </c>
       <c r="I1" t="s">
-        <v>169</v>
+        <v>117</v>
       </c>
       <c r="J1" t="s">
-        <v>178</v>
+        <v>126</v>
       </c>
       <c r="K1" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="2">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -645,7 +946,7 @@
         <v>10</v>
       </c>
       <c r="D2">
-        <v>0.100000001490116</v>
+        <v>0.10000000149011599</v>
       </c>
       <c r="E2">
         <v>8000</v>
@@ -657,7 +958,7 @@
         <v>350</v>
       </c>
       <c r="H2" t="s">
-        <v>170</v>
+        <v>118</v>
       </c>
       <c r="I2">
         <v>5000</v>
@@ -669,18 +970,18 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" t="s">
         <v>12</v>
-      </c>
-      <c r="B3" t="s">
-        <v>13</v>
       </c>
       <c r="C3" t="s">
         <v>10</v>
       </c>
       <c r="D3">
-        <v>0.0500000007450581</v>
+        <v>5.0000000745058101E-2</v>
       </c>
       <c r="E3">
         <v>9999</v>
@@ -692,27 +993,27 @@
         <v>25</v>
       </c>
       <c r="H3" t="s">
-        <v>171</v>
+        <v>119</v>
       </c>
       <c r="I3">
         <v>5000</v>
       </c>
       <c r="J3">
-        <v>3.05999994277954</v>
+        <v>3.0599999427795401</v>
       </c>
       <c r="K3">
         <v>7</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D4">
         <v>8</v>
@@ -727,27 +1028,27 @@
         <v>45</v>
       </c>
       <c r="H4" t="s">
-        <v>172</v>
+        <v>120</v>
       </c>
       <c r="I4">
         <v>20</v>
       </c>
       <c r="J4">
-        <v>2.10999989509583</v>
+        <v>2.1099998950958301</v>
       </c>
       <c r="K4">
         <v>3</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D5">
         <v>10</v>
@@ -762,27 +1063,27 @@
         <v>20</v>
       </c>
       <c r="H5" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I5">
         <v>20</v>
       </c>
       <c r="J5">
-        <v>0.449999988079071</v>
+        <v>0.44999998807907099</v>
       </c>
       <c r="K5">
         <v>2</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B6" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C6" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D6">
         <v>4</v>
@@ -797,7 +1098,7 @@
         <v>60</v>
       </c>
       <c r="H6" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I6">
         <v>80</v>
@@ -809,15 +1110,15 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="B7" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="C7" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D7">
         <v>0.5</v>
@@ -832,7 +1133,7 @@
         <v>220</v>
       </c>
       <c r="H7" t="s">
-        <v>174</v>
+        <v>122</v>
       </c>
       <c r="I7">
         <v>1000</v>
@@ -844,15 +1145,15 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="B8" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="C8" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D8">
         <v>5</v>
@@ -867,27 +1168,27 @@
         <v>70</v>
       </c>
       <c r="H8" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I8">
         <v>80</v>
       </c>
       <c r="J8">
-        <v>6.65999984741211</v>
+        <v>6.6599998474121103</v>
       </c>
       <c r="K8">
         <v>4</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B9" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="C9" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D9">
         <v>7</v>
@@ -902,27 +1203,27 @@
         <v>80</v>
       </c>
       <c r="H9" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I9">
         <v>20</v>
       </c>
       <c r="J9">
-        <v>7.19999980926514</v>
+        <v>7.1999998092651403</v>
       </c>
       <c r="K9">
         <v>3</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="B10" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="C10" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D10">
         <v>6</v>
@@ -937,27 +1238,27 @@
         <v>15</v>
       </c>
       <c r="H10" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I10">
         <v>20</v>
       </c>
       <c r="J10">
-        <v>0.200000002980232</v>
+        <v>0.20000000298023199</v>
       </c>
       <c r="K10">
         <v>2</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="B11" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="C11" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D11">
         <v>9</v>
@@ -972,27 +1273,27 @@
         <v>25</v>
       </c>
       <c r="H11" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I11">
         <v>20</v>
       </c>
       <c r="J11">
-        <v>0.800000011920929</v>
+        <v>0.80000001192092896</v>
       </c>
       <c r="K11">
         <v>2</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="B12" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="C12" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D12">
         <v>8.5</v>
@@ -1007,7 +1308,7 @@
         <v>10</v>
       </c>
       <c r="H12" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I12">
         <v>20</v>
@@ -1019,15 +1320,15 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="B13" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="C13" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D13">
         <v>3.5</v>
@@ -1042,27 +1343,27 @@
         <v>50</v>
       </c>
       <c r="H13" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I13">
         <v>80</v>
       </c>
       <c r="J13">
-        <v>3.08999991416931</v>
+        <v>3.0899999141693102</v>
       </c>
       <c r="K13">
         <v>4</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="B14" t="s">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="C14" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D14">
         <v>10</v>
@@ -1077,27 +1378,27 @@
         <v>8</v>
       </c>
       <c r="H14" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I14">
         <v>20</v>
       </c>
       <c r="J14">
-        <v>0.0599999986588955</v>
+        <v>5.9999998658895499E-2</v>
       </c>
       <c r="K14">
         <v>2</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="B15" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="C15" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="D15">
         <v>1.5</v>
@@ -1112,30 +1413,30 @@
         <v>150</v>
       </c>
       <c r="H15" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I15">
         <v>250</v>
       </c>
       <c r="J15">
-        <v>39.6800003051758</v>
+        <v>39.680000305175803</v>
       </c>
       <c r="K15">
         <v>6</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>55</v>
+        <v>41</v>
       </c>
       <c r="B16" t="s">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="C16" t="s">
         <v>10</v>
       </c>
       <c r="D16">
-        <v>0.100000001490116</v>
+        <v>0.10000000149011599</v>
       </c>
       <c r="E16">
         <v>7777</v>
@@ -1147,7 +1448,7 @@
         <v>50</v>
       </c>
       <c r="H16" t="s">
-        <v>172</v>
+        <v>120</v>
       </c>
       <c r="I16">
         <v>5000</v>
@@ -1159,15 +1460,15 @@
         <v>8</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>58</v>
+        <v>43</v>
       </c>
       <c r="B17" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="C17" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D17">
         <v>5</v>
@@ -1182,27 +1483,27 @@
         <v>15</v>
       </c>
       <c r="H17" t="s">
-        <v>175</v>
+        <v>123</v>
       </c>
       <c r="I17">
         <v>20</v>
       </c>
       <c r="J17">
-        <v>0.200000002980232</v>
+        <v>0.20000000298023199</v>
       </c>
       <c r="K17">
         <v>2</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="B18" t="s">
-        <v>62</v>
+        <v>46</v>
       </c>
       <c r="C18" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D18">
         <v>12</v>
@@ -1217,30 +1518,30 @@
         <v>5</v>
       </c>
       <c r="H18" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I18">
         <v>20</v>
       </c>
       <c r="J18">
-        <v>0.0199999995529652</v>
+        <v>1.9999999552965199E-2</v>
       </c>
       <c r="K18">
         <v>2</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>64</v>
+        <v>47</v>
       </c>
       <c r="B19" t="s">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="C19" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D19">
-        <v>0.800000011920929</v>
+        <v>0.80000001192092896</v>
       </c>
       <c r="E19">
         <v>2500</v>
@@ -1252,7 +1553,7 @@
         <v>120</v>
       </c>
       <c r="H19" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I19">
         <v>1000</v>
@@ -1264,15 +1565,15 @@
         <v>8</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="B20" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
       <c r="C20" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="D20">
         <v>2</v>
@@ -1287,27 +1588,27 @@
         <v>65</v>
       </c>
       <c r="H20" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I20">
         <v>250</v>
       </c>
       <c r="J20">
-        <v>6.76999998092651</v>
+        <v>6.7699999809265101</v>
       </c>
       <c r="K20">
         <v>5</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>70</v>
+        <v>51</v>
       </c>
       <c r="B21" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="C21" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D21">
         <v>10</v>
@@ -1322,27 +1623,27 @@
         <v>5</v>
       </c>
       <c r="H21" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I21">
         <v>20</v>
       </c>
       <c r="J21">
-        <v>0.0199999995529652</v>
+        <v>1.9999999552965199E-2</v>
       </c>
       <c r="K21">
         <v>2</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>73</v>
+        <v>53</v>
       </c>
       <c r="B22" t="s">
-        <v>74</v>
+        <v>54</v>
       </c>
       <c r="C22" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D22">
         <v>3</v>
@@ -1357,27 +1658,27 @@
         <v>30</v>
       </c>
       <c r="H22" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I22">
         <v>80</v>
       </c>
       <c r="J22">
-        <v>1.11000001430511</v>
+        <v>1.1100000143051101</v>
       </c>
       <c r="K22">
         <v>3</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>76</v>
+        <v>55</v>
       </c>
       <c r="B23" t="s">
-        <v>77</v>
+        <v>56</v>
       </c>
       <c r="C23" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="D23">
         <v>1.20000004768372</v>
@@ -1392,7 +1693,7 @@
         <v>130</v>
       </c>
       <c r="H23" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I23">
         <v>250</v>
@@ -1404,15 +1705,15 @@
         <v>6</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>79</v>
+        <v>57</v>
       </c>
       <c r="B24" t="s">
-        <v>80</v>
+        <v>58</v>
       </c>
       <c r="C24" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D24">
         <v>8</v>
@@ -1427,7 +1728,7 @@
         <v>35</v>
       </c>
       <c r="H24" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I24">
         <v>20</v>
@@ -1439,15 +1740,15 @@
         <v>3</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>82</v>
+        <v>59</v>
       </c>
       <c r="B25" t="s">
-        <v>83</v>
+        <v>60</v>
       </c>
       <c r="C25" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="D25">
         <v>2.5</v>
@@ -1462,30 +1763,30 @@
         <v>100</v>
       </c>
       <c r="H25" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I25">
         <v>250</v>
       </c>
       <c r="J25">
-        <v>16.8799991607666</v>
+        <v>16.879999160766602</v>
       </c>
       <c r="K25">
         <v>6</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>85</v>
+        <v>61</v>
       </c>
       <c r="B26" t="s">
-        <v>86</v>
+        <v>62</v>
       </c>
       <c r="C26" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D26">
-        <v>0.200000002980232</v>
+        <v>0.20000000298023199</v>
       </c>
       <c r="E26">
         <v>5000</v>
@@ -1497,27 +1798,27 @@
         <v>4</v>
       </c>
       <c r="H26" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I26">
         <v>20</v>
       </c>
       <c r="J26">
-        <v>0.00999999977648258</v>
+        <v>9.9999997764825804E-3</v>
       </c>
       <c r="K26">
         <v>2</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>88</v>
+        <v>63</v>
       </c>
       <c r="B27" t="s">
-        <v>89</v>
+        <v>64</v>
       </c>
       <c r="C27" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="D27">
         <v>3</v>
@@ -1532,27 +1833,27 @@
         <v>55</v>
       </c>
       <c r="H27" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I27">
         <v>250</v>
       </c>
       <c r="J27">
-        <v>5.42000007629395</v>
+        <v>5.4200000762939498</v>
       </c>
       <c r="K27">
         <v>5</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>91</v>
+        <v>65</v>
       </c>
       <c r="B28" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="C28" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D28">
         <v>4.5</v>
@@ -1567,27 +1868,27 @@
         <v>80</v>
       </c>
       <c r="H28" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I28">
         <v>80</v>
       </c>
       <c r="J28">
-        <v>7.92000007629395</v>
+        <v>7.9200000762939498</v>
       </c>
       <c r="K28">
         <v>4</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>94</v>
+        <v>67</v>
       </c>
       <c r="B29" t="s">
-        <v>95</v>
+        <v>68</v>
       </c>
       <c r="C29" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D29">
         <v>15</v>
@@ -1602,30 +1903,30 @@
         <v>3</v>
       </c>
       <c r="H29" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I29">
         <v>20</v>
       </c>
       <c r="J29">
-        <v>0.00999999977648258</v>
+        <v>9.9999997764825804E-3</v>
       </c>
       <c r="K29">
         <v>2</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>97</v>
+        <v>69</v>
       </c>
       <c r="B30" t="s">
-        <v>98</v>
+        <v>70</v>
       </c>
       <c r="C30" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D30">
-        <v>0.400000005960464</v>
+        <v>0.40000000596046398</v>
       </c>
       <c r="E30">
         <v>4500</v>
@@ -1637,27 +1938,27 @@
         <v>250</v>
       </c>
       <c r="H30" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I30">
         <v>1000</v>
       </c>
       <c r="J30">
-        <v>153.119995117188</v>
+        <v>153.11999511718801</v>
       </c>
       <c r="K30">
         <v>8</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>100</v>
+        <v>71</v>
       </c>
       <c r="B31" t="s">
-        <v>101</v>
+        <v>72</v>
       </c>
       <c r="C31" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D31">
         <v>7</v>
@@ -1672,7 +1973,7 @@
         <v>12</v>
       </c>
       <c r="H31" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I31">
         <v>20</v>
@@ -1684,15 +1985,15 @@
         <v>2</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>103</v>
+        <v>73</v>
       </c>
       <c r="B32" t="s">
-        <v>104</v>
+        <v>74</v>
       </c>
       <c r="C32" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D32">
         <v>2</v>
@@ -1707,7 +2008,7 @@
         <v>40</v>
       </c>
       <c r="H32" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I32">
         <v>80</v>
@@ -1719,18 +2020,18 @@
         <v>4</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>106</v>
+        <v>75</v>
       </c>
       <c r="B33" t="s">
-        <v>107</v>
+        <v>76</v>
       </c>
       <c r="C33" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="D33">
-        <v>3.79999995231628</v>
+        <v>3.7999999523162802</v>
       </c>
       <c r="E33">
         <v>450</v>
@@ -1742,27 +2043,27 @@
         <v>60</v>
       </c>
       <c r="H33" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I33">
         <v>250</v>
       </c>
       <c r="J33">
-        <v>6.07999992370605</v>
+        <v>6.0799999237060502</v>
       </c>
       <c r="K33">
         <v>5</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>109</v>
+        <v>77</v>
       </c>
       <c r="B34" t="s">
-        <v>110</v>
+        <v>78</v>
       </c>
       <c r="C34" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D34">
         <v>4</v>
@@ -1777,7 +2078,7 @@
         <v>20</v>
       </c>
       <c r="H34" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I34">
         <v>1000</v>
@@ -1789,15 +2090,15 @@
         <v>5</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>112</v>
+        <v>79</v>
       </c>
       <c r="B35" t="s">
-        <v>113</v>
+        <v>80</v>
       </c>
       <c r="C35" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D35">
         <v>7.5</v>
@@ -1812,27 +2113,27 @@
         <v>50</v>
       </c>
       <c r="H35" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I35">
         <v>20</v>
       </c>
       <c r="J35">
-        <v>2.80999994277954</v>
+        <v>2.8099999427795401</v>
       </c>
       <c r="K35">
         <v>3</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
       <c r="B36" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="C36" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D36">
         <v>5.5</v>
@@ -1847,7 +2148,7 @@
         <v>10</v>
       </c>
       <c r="H36" t="s">
-        <v>176</v>
+        <v>124</v>
       </c>
       <c r="I36">
         <v>20</v>
@@ -1859,18 +2160,18 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>118</v>
+        <v>83</v>
       </c>
       <c r="B37" t="s">
-        <v>119</v>
+        <v>84</v>
       </c>
       <c r="C37" t="s">
         <v>10</v>
       </c>
       <c r="D37">
-        <v>0.0799999982118607</v>
+        <v>7.9999998211860698E-2</v>
       </c>
       <c r="E37">
         <v>12000</v>
@@ -1882,7 +2183,7 @@
         <v>180</v>
       </c>
       <c r="H37" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I37">
         <v>5000</v>
@@ -1894,18 +2195,18 @@
         <v>9</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>121</v>
+        <v>85</v>
       </c>
       <c r="B38" t="s">
-        <v>122</v>
+        <v>86</v>
       </c>
       <c r="C38" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D38">
-        <v>3.20000004768372</v>
+        <v>3.2000000476837198</v>
       </c>
       <c r="E38">
         <v>550</v>
@@ -1917,7 +2218,7 @@
         <v>100</v>
       </c>
       <c r="H38" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I38">
         <v>80</v>
@@ -1929,18 +2230,18 @@
         <v>5</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>124</v>
+        <v>87</v>
       </c>
       <c r="B39" t="s">
-        <v>125</v>
+        <v>88</v>
       </c>
       <c r="C39" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D39">
-        <v>2.20000004768372</v>
+        <v>2.2000000476837198</v>
       </c>
       <c r="E39">
         <v>1100</v>
@@ -1952,30 +2253,30 @@
         <v>110</v>
       </c>
       <c r="H39" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I39">
         <v>20</v>
       </c>
       <c r="J39">
-        <v>14.4499998092651</v>
+        <v>14.449999809265099</v>
       </c>
       <c r="K39">
         <v>4</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>127</v>
+        <v>89</v>
       </c>
       <c r="B40" t="s">
-        <v>128</v>
+        <v>90</v>
       </c>
       <c r="C40" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D40">
-        <v>8.19999980926514</v>
+        <v>8.1999998092651403</v>
       </c>
       <c r="E40">
         <v>220</v>
@@ -1987,7 +2288,7 @@
         <v>40</v>
       </c>
       <c r="H40" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I40">
         <v>20</v>
@@ -1999,15 +2300,15 @@
         <v>3</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>130</v>
+        <v>91</v>
       </c>
       <c r="B41" t="s">
-        <v>131</v>
+        <v>92</v>
       </c>
       <c r="C41" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="D41">
         <v>1.79999995231628</v>
@@ -2022,27 +2323,27 @@
         <v>150</v>
       </c>
       <c r="H41" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I41">
         <v>250</v>
       </c>
       <c r="J41">
-        <v>39.6800003051758</v>
+        <v>39.680000305175803</v>
       </c>
       <c r="K41">
         <v>6</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>133</v>
+        <v>93</v>
       </c>
       <c r="B42" t="s">
-        <v>134</v>
+        <v>94</v>
       </c>
       <c r="C42" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D42">
         <v>11</v>
@@ -2057,27 +2358,27 @@
         <v>30</v>
       </c>
       <c r="H42" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I42">
         <v>20</v>
       </c>
       <c r="J42">
-        <v>1.00999999046326</v>
+        <v>1.0099999904632599</v>
       </c>
       <c r="K42">
         <v>2</v>
       </c>
     </row>
-    <row r="43">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>136</v>
+        <v>95</v>
       </c>
       <c r="B43" t="s">
-        <v>137</v>
+        <v>96</v>
       </c>
       <c r="C43" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D43">
         <v>20</v>
@@ -2092,7 +2393,7 @@
         <v>2</v>
       </c>
       <c r="H43" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I43">
         <v>20</v>
@@ -2104,15 +2405,15 @@
         <v>2</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>139</v>
+        <v>97</v>
       </c>
       <c r="B44" t="s">
-        <v>140</v>
+        <v>98</v>
       </c>
       <c r="C44" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="D44">
         <v>2</v>
@@ -2127,7 +2428,7 @@
         <v>35</v>
       </c>
       <c r="H44" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I44">
         <v>250</v>
@@ -2139,15 +2440,15 @@
         <v>5</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>142</v>
+        <v>99</v>
       </c>
       <c r="B45" t="s">
-        <v>143</v>
+        <v>100</v>
       </c>
       <c r="C45" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D45">
         <v>1</v>
@@ -2162,30 +2463,30 @@
         <v>45</v>
       </c>
       <c r="H45" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I45">
         <v>1000</v>
       </c>
       <c r="J45">
-        <v>5.28000020980835</v>
+        <v>5.2800002098083496</v>
       </c>
       <c r="K45">
         <v>6</v>
       </c>
     </row>
-    <row r="46">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>145</v>
+        <v>101</v>
       </c>
       <c r="B46" t="s">
-        <v>146</v>
+        <v>102</v>
       </c>
       <c r="C46" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D46">
-        <v>0.699999988079071</v>
+        <v>0.69999998807907104</v>
       </c>
       <c r="E46">
         <v>5500</v>
@@ -2197,27 +2498,27 @@
         <v>30</v>
       </c>
       <c r="H46" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I46">
         <v>1000</v>
       </c>
       <c r="J46">
-        <v>2.52999997138977</v>
+        <v>2.5299999713897701</v>
       </c>
       <c r="K46">
         <v>6</v>
       </c>
     </row>
-    <row r="47">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>148</v>
+        <v>103</v>
       </c>
       <c r="B47" t="s">
-        <v>149</v>
+        <v>104</v>
       </c>
       <c r="C47" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="D47">
         <v>1.5</v>
@@ -2232,30 +2533,30 @@
         <v>250</v>
       </c>
       <c r="H47" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I47">
         <v>250</v>
       </c>
       <c r="J47">
-        <v>91.879997253418</v>
+        <v>91.879997253417997</v>
       </c>
       <c r="K47">
         <v>7</v>
       </c>
     </row>
-    <row r="48">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>151</v>
+        <v>105</v>
       </c>
       <c r="B48" t="s">
-        <v>152</v>
+        <v>106</v>
       </c>
       <c r="C48" t="s">
         <v>10</v>
       </c>
       <c r="D48">
-        <v>0.0500000007450581</v>
+        <v>5.0000000745058101E-2</v>
       </c>
       <c r="E48">
         <v>15000</v>
@@ -2267,7 +2568,7 @@
         <v>300</v>
       </c>
       <c r="H48" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I48">
         <v>5000</v>
@@ -2279,18 +2580,18 @@
         <v>10</v>
       </c>
     </row>
-    <row r="49">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>154</v>
+        <v>107</v>
       </c>
       <c r="B49" t="s">
-        <v>155</v>
+        <v>108</v>
       </c>
       <c r="C49" t="s">
         <v>10</v>
       </c>
       <c r="D49">
-        <v>0.150000005960464</v>
+        <v>0.15000000596046401</v>
       </c>
       <c r="E49">
         <v>9000</v>
@@ -2302,7 +2603,7 @@
         <v>120</v>
       </c>
       <c r="H49" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I49">
         <v>5000</v>
@@ -2314,18 +2615,18 @@
         <v>9</v>
       </c>
     </row>
-    <row r="50">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>157</v>
+        <v>109</v>
       </c>
       <c r="B50" t="s">
-        <v>158</v>
+        <v>110</v>
       </c>
       <c r="C50" t="s">
         <v>10</v>
       </c>
       <c r="D50">
-        <v>0.0500000007450581</v>
+        <v>5.0000000745058101E-2</v>
       </c>
       <c r="E50">
         <v>25000</v>
@@ -2337,7 +2638,7 @@
         <v>100</v>
       </c>
       <c r="H50" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I50">
         <v>5000</v>
@@ -2349,18 +2650,18 @@
         <v>9</v>
       </c>
     </row>
-    <row r="51">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>160</v>
+        <v>111</v>
       </c>
       <c r="B51" t="s">
-        <v>161</v>
+        <v>112</v>
       </c>
       <c r="C51" t="s">
         <v>10</v>
       </c>
       <c r="D51">
-        <v>0.0500000007450581</v>
+        <v>5.0000000745058101E-2</v>
       </c>
       <c r="E51">
         <v>30000</v>
@@ -2372,7 +2673,7 @@
         <v>400</v>
       </c>
       <c r="H51" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I51">
         <v>5000</v>
@@ -2384,18 +2685,18 @@
         <v>10</v>
       </c>
     </row>
-    <row r="52">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>163</v>
+        <v>113</v>
       </c>
       <c r="B52" t="s">
-        <v>164</v>
+        <v>114</v>
       </c>
       <c r="C52" t="s">
         <v>10</v>
       </c>
       <c r="D52">
-        <v>0.0199999995529652</v>
+        <v>1.9999999552965199E-2</v>
       </c>
       <c r="E52">
         <v>45000</v>
@@ -2407,7 +2708,7 @@
         <v>1600</v>
       </c>
       <c r="H52" t="s">
-        <v>173</v>
+        <v>121</v>
       </c>
       <c r="I52">
         <v>5000</v>
@@ -2419,18 +2720,18 @@
         <v>10</v>
       </c>
     </row>
-    <row r="53">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>166</v>
+        <v>115</v>
       </c>
       <c r="B53" t="s">
-        <v>167</v>
+        <v>116</v>
       </c>
       <c r="C53" t="s">
         <v>10</v>
       </c>
       <c r="D53">
-        <v>0.00999999977648258</v>
+        <v>9.9999997764825804E-3</v>
       </c>
       <c r="E53">
         <v>99999</v>
@@ -2442,7 +2743,7 @@
         <v>500</v>
       </c>
       <c r="H53" t="s">
-        <v>177</v>
+        <v>125</v>
       </c>
       <c r="I53">
         <v>5000</v>
@@ -2455,6 +2756,346 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr defaultColWidth="8.375" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>128</v>
+      </c>
+      <c r="E1" t="s">
+        <v>129</v>
+      </c>
+      <c r="F1" t="s">
+        <v>130</v>
+      </c>
+      <c r="G1" t="s">
+        <v>131</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B2" t="s">
+        <v>133</v>
+      </c>
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>100</v>
+      </c>
+      <c r="H2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>135</v>
+      </c>
+      <c r="B3" t="s">
+        <v>136</v>
+      </c>
+      <c r="C3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3">
+        <v>3000</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3">
+        <v>3</v>
+      </c>
+      <c r="G3">
+        <v>150</v>
+      </c>
+      <c r="H3" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>138</v>
+      </c>
+      <c r="B4" t="s">
+        <v>139</v>
+      </c>
+      <c r="C4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D4">
+        <v>8000</v>
+      </c>
+      <c r="E4">
+        <v>5</v>
+      </c>
+      <c r="F4">
+        <v>5</v>
+      </c>
+      <c r="G4">
+        <v>200</v>
+      </c>
+      <c r="H4" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>141</v>
+      </c>
+      <c r="B5" t="s">
+        <v>142</v>
+      </c>
+      <c r="C5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5">
+        <v>20000</v>
+      </c>
+      <c r="E5">
+        <v>10</v>
+      </c>
+      <c r="F5">
+        <v>8</v>
+      </c>
+      <c r="G5">
+        <v>300</v>
+      </c>
+      <c r="H5" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>144</v>
+      </c>
+      <c r="B6" t="s">
+        <v>145</v>
+      </c>
+      <c r="C6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6">
+        <v>50000</v>
+      </c>
+      <c r="E6">
+        <v>15</v>
+      </c>
+      <c r="F6">
+        <v>15</v>
+      </c>
+      <c r="G6">
+        <v>500</v>
+      </c>
+      <c r="H6" t="s">
+        <v>146</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr defaultColWidth="8.375" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>128</v>
+      </c>
+      <c r="E1" t="s">
+        <v>147</v>
+      </c>
+      <c r="F1" t="s">
+        <v>130</v>
+      </c>
+      <c r="G1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B2" t="s">
+        <v>149</v>
+      </c>
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2" t="s">
+        <v>150</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>152</v>
+      </c>
+      <c r="B3" t="s">
+        <v>153</v>
+      </c>
+      <c r="C3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3">
+        <v>500</v>
+      </c>
+      <c r="E3" t="s">
+        <v>154</v>
+      </c>
+      <c r="F3">
+        <v>5</v>
+      </c>
+      <c r="G3" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>156</v>
+      </c>
+      <c r="B4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4">
+        <v>600</v>
+      </c>
+      <c r="E4" t="s">
+        <v>158</v>
+      </c>
+      <c r="F4">
+        <v>5</v>
+      </c>
+      <c r="G4" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>160</v>
+      </c>
+      <c r="B5" t="s">
+        <v>161</v>
+      </c>
+      <c r="C5" t="s">
+        <v>40</v>
+      </c>
+      <c r="D5">
+        <v>2000</v>
+      </c>
+      <c r="E5" t="s">
+        <v>150</v>
+      </c>
+      <c r="F5">
+        <v>10</v>
+      </c>
+      <c r="G5" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>163</v>
+      </c>
+      <c r="B6" t="s">
+        <v>164</v>
+      </c>
+      <c r="C6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6">
+        <v>8000</v>
+      </c>
+      <c r="E6" t="s">
+        <v>165</v>
+      </c>
+      <c r="F6">
+        <v>20</v>
+      </c>
+      <c r="G6" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>167</v>
+      </c>
+      <c r="B7" t="s">
+        <v>168</v>
+      </c>
+      <c r="C7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7">
+        <v>20000</v>
+      </c>
+      <c r="E7" t="s">
+        <v>169</v>
+      </c>
+      <c r="F7">
+        <v>30</v>
+      </c>
+      <c r="G7" t="s">
+        <v>170</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: integrate inventory, shop, and rod views with TopTapGroup switching
- InventoryUI: view switching via TopTapGroup (인벤/샵/로즈)
- SideTabs and rank filter removed, simplified to tab-based navigation
- Shop view: all Excel fish catalog with buy button
- Rods view: 5 rods (basic/carbon/fiberglass/titanium/legendary) with buy/equip/unequip
- Rod icons added to Assets/Art/Rods/
- RodIconMatcher editor tool for assigning rod sprites
- ExcelDataConverter: ghost fish cleanup on conversion
- Fish descriptions added for all Excel species
- FishIconMatcher: fixed icon mapping for missing sprites
- FishingController: block input when inventory open (cursor check)
- UserStorageService: ghost data cleanup on load, default rod_basic granted
- NetworkMenuUI: SetVisible() + disable component when inventory open
</commit_message>
<xml_diff>
--- a/Assets/ExcelData/FishData.xlsx
+++ b/Assets/ExcelData/FishData.xlsx
@@ -3,14 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Unity\MultiplayFishingGame\Assets\ExcelData\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_CF4A63481BB9D411202F87246475D13240D807F7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3075" yWindow="3075" windowWidth="21600" windowHeight="11385" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3075" yWindow="3075" windowWidth="21600" windowHeight="11385"/>
   </bookViews>
   <sheets>
     <sheet name="FishList" sheetId="1" r:id="rId1"/>
@@ -22,525 +16,682 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="171">
-  <si>
-    <t>ID</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>Rank</t>
-  </si>
-  <si>
-    <t>Chance (%)</t>
-  </si>
-  <si>
-    <t>Price (Gold)</t>
-  </si>
-  <si>
-    <t>Min Length (cm)</t>
-  </si>
-  <si>
-    <t>Max Length (cm)</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>fish_alligator</t>
-  </si>
-  <si>
-    <t>악어</t>
-  </si>
-  <si>
-    <t>★★★★★</t>
-  </si>
-  <si>
-    <t>fish_axolotl</t>
-  </si>
-  <si>
-    <t>아홀로틀</t>
-  </si>
-  <si>
-    <t>fish_bass</t>
-  </si>
-  <si>
-    <t>큰입배스</t>
-  </si>
-  <si>
-    <t>★</t>
-  </si>
-  <si>
-    <t>fish_bluegill</t>
-  </si>
-  <si>
-    <t>블루길</t>
-  </si>
-  <si>
-    <t>fish_bowfin</t>
-  </si>
-  <si>
-    <t>보우핀</t>
-  </si>
-  <si>
-    <t>★★</t>
-  </si>
-  <si>
-    <t>fish_bullshark</t>
-  </si>
-  <si>
-    <t>황소상어</t>
-  </si>
-  <si>
-    <t>★★★★</t>
-  </si>
-  <si>
-    <t>fish_carp</t>
-  </si>
-  <si>
-    <t>잉어</t>
-  </si>
-  <si>
-    <t>fish_catfish</t>
-  </si>
-  <si>
-    <t>메기</t>
-  </si>
-  <si>
-    <t>fish_crab</t>
-  </si>
-  <si>
-    <t>게</t>
-  </si>
-  <si>
-    <t>fish_crappie</t>
-  </si>
-  <si>
-    <t>크래피</t>
-  </si>
-  <si>
-    <t>fish_crayfish</t>
-  </si>
-  <si>
-    <t>가재</t>
-  </si>
-  <si>
-    <t>fish_drum</t>
-  </si>
-  <si>
-    <t>민어</t>
-  </si>
-  <si>
-    <t>fish_frog</t>
-  </si>
-  <si>
-    <t>개구리</t>
-  </si>
-  <si>
-    <t>fish_gar</t>
-  </si>
-  <si>
-    <t>가아</t>
-  </si>
-  <si>
-    <t>★★★</t>
-  </si>
-  <si>
-    <t>fish_bass_golden</t>
-  </si>
-  <si>
-    <t>골든 배스</t>
-  </si>
-  <si>
-    <t>fish_goldfish</t>
-  </si>
-  <si>
-    <t>금붕어</t>
-  </si>
-  <si>
-    <t>fish_guppy</t>
-  </si>
-  <si>
-    <t>구피</t>
-  </si>
-  <si>
-    <t>fish_salmon_king</t>
-  </si>
-  <si>
-    <t>왕연어</t>
-  </si>
-  <si>
-    <t>fish_koi</t>
-  </si>
-  <si>
-    <t>비단잉어</t>
-  </si>
-  <si>
-    <t>fish_leech</t>
-  </si>
-  <si>
-    <t>거머리</t>
-  </si>
-  <si>
-    <t>fish_mooneye</t>
-  </si>
-  <si>
-    <t>문아이</t>
-  </si>
-  <si>
-    <t>fish_muskellunge</t>
-  </si>
-  <si>
-    <t>머스키</t>
-  </si>
-  <si>
-    <t>fish_perch</t>
-  </si>
-  <si>
-    <t>퍼치</t>
-  </si>
-  <si>
-    <t>fish_pike</t>
-  </si>
-  <si>
-    <t>강꼬치고기</t>
-  </si>
-  <si>
-    <t>fish_pupfish</t>
-  </si>
-  <si>
-    <t>펍피쉬</t>
-  </si>
-  <si>
-    <t>fish_trout_rainbow</t>
-  </si>
-  <si>
-    <t>무지개송어</t>
-  </si>
-  <si>
-    <t>fish_salmon</t>
-  </si>
-  <si>
-    <t>연어</t>
-  </si>
-  <si>
-    <t>fish_snail</t>
-  </si>
-  <si>
-    <t>달팽이</t>
-  </si>
-  <si>
-    <t>fish_sturgeon</t>
-  </si>
-  <si>
-    <t>철갑상어</t>
-  </si>
-  <si>
-    <t>fish_toad</t>
-  </si>
-  <si>
-    <t>두꺼비</t>
-  </si>
-  <si>
-    <t>fish_turtle</t>
-  </si>
-  <si>
-    <t>거북이</t>
-  </si>
-  <si>
-    <t>fish_walleye</t>
-  </si>
-  <si>
-    <t>월아이</t>
-  </si>
-  <si>
-    <t>fish_angelfish</t>
-  </si>
-  <si>
-    <t>엔젤피쉬</t>
-  </si>
-  <si>
-    <t>fish_bluefish</t>
-  </si>
-  <si>
-    <t>블루피쉬</t>
-  </si>
-  <si>
-    <t>fish_clownfish</t>
-  </si>
-  <si>
-    <t>흰동가리</t>
-  </si>
-  <si>
-    <t>fish_coelacanth</t>
-  </si>
-  <si>
-    <t>실러캔스</t>
-  </si>
-  <si>
-    <t>fish_dogfish</t>
-  </si>
-  <si>
-    <t>돔발상어</t>
-  </si>
-  <si>
-    <t>fish_eel</t>
-  </si>
-  <si>
-    <t>장어</t>
-  </si>
-  <si>
-    <t>fish_flounder</t>
-  </si>
-  <si>
-    <t>가자미</t>
-  </si>
-  <si>
-    <t>fish_grouper</t>
-  </si>
-  <si>
-    <t>그루퍼</t>
-  </si>
-  <si>
-    <t>fish_herring</t>
-  </si>
-  <si>
-    <t>청어</t>
-  </si>
-  <si>
-    <t>fish_krill</t>
-  </si>
-  <si>
-    <t>크릴</t>
-  </si>
-  <si>
-    <t>fish_lionfish</t>
-  </si>
-  <si>
-    <t>쏠배감펭</t>
-  </si>
-  <si>
-    <t>fish_lobster</t>
-  </si>
-  <si>
-    <t>바닷가재</t>
-  </si>
-  <si>
-    <t>fish_manowar</t>
-  </si>
-  <si>
-    <t>만오워</t>
-  </si>
-  <si>
-    <t>fish_mantaray</t>
-  </si>
-  <si>
-    <t>가오리</t>
-  </si>
-  <si>
-    <t>fish_mantaray_golden</t>
-  </si>
-  <si>
-    <t>황금 가오리</t>
-  </si>
-  <si>
-    <t>fish_seaturtle</t>
-  </si>
-  <si>
-    <t>바다거북</t>
-  </si>
-  <si>
-    <t>fish_anomalocaris</t>
-  </si>
-  <si>
-    <t>아노말로카리스</t>
-  </si>
-  <si>
-    <t>fish_helicoprion</t>
-  </si>
-  <si>
-    <t>헬리코프리온</t>
-  </si>
-  <si>
-    <t>fish_leedsichthys</t>
-  </si>
-  <si>
-    <t>리드시크티스</t>
-  </si>
-  <si>
-    <t>fish_ufo</t>
-  </si>
-  <si>
-    <t>UFO</t>
-  </si>
-  <si>
-    <t>EXP Reward</t>
-  </si>
-  <si>
-    <t>강의 지배자. 날카로운 이빨을 조심하세요.</t>
-  </si>
-  <si>
-    <t>웃는 얼굴의 귀여운 도롱뇽. 보고만 있어도 기분이 좋아집니다.</t>
-  </si>
-  <si>
-    <t>입이 정말 커서 무엇이든 집어삼키는 탐욕스러운 물고기입니다.</t>
-  </si>
-  <si>
-    <t>평범하지만 특별한 당신만의 물고기입니다.</t>
-  </si>
-  <si>
-    <t>바다의 최상위 포식자. 잡았다는 것 자체가 기적입니다!</t>
-  </si>
-  <si>
-    <t>어항에서 탈출한 걸까요? 반짝이는 비늘이 아름답습니다.</t>
-  </si>
-  <si>
-    <t>산호초 사이를 헤엄치는 귀여운 물고기. 영화 속 주인공 같아요.</t>
-  </si>
-  <si>
-    <t>이건 물고기가 아닙니다! 외계에서 날아온 비행 물체네요.</t>
-  </si>
-  <si>
-    <t>Weight</t>
-  </si>
-  <si>
-    <t>Required Spam</t>
-  </si>
-  <si>
-    <t>Price</t>
-  </si>
-  <si>
-    <t>CastDistanceBonus</t>
-  </si>
-  <si>
-    <t>CatchChanceBonus</t>
-  </si>
-  <si>
-    <t>Durability</t>
-  </si>
-  <si>
-    <t>rod_basic</t>
-  </si>
-  <si>
-    <t>기본 낚싯대</t>
-  </si>
-  <si>
-    <t>누구나 사용할 수 있는 기본 낚싯대입니다.</t>
-  </si>
-  <si>
-    <t>rod_carbon</t>
-  </si>
-  <si>
-    <t>카본 낚싯대</t>
-  </si>
-  <si>
-    <t>가볍고 튼튼한 카본 소재의 낚싯대입니다.</t>
-  </si>
-  <si>
-    <t>rod_fiberglass</t>
-  </si>
-  <si>
-    <t>유리섬유 낚싯대</t>
-  </si>
-  <si>
-    <t>유리섬유 소재로 제작된 중급 낚싯대입니다.</t>
-  </si>
-  <si>
-    <t>rod_titanium</t>
-  </si>
-  <si>
-    <t>티타늄 낚싯대</t>
-  </si>
-  <si>
-    <t>초경량 티타늄 합금으로 제작된 고급 낚싯대입니다.</t>
-  </si>
-  <si>
-    <t>rod_legendary</t>
-  </si>
-  <si>
-    <t>전설의 낚싯대</t>
-  </si>
-  <si>
-    <t>전설 속에만 존재한다는 궁극의 낚싯대입니다.</t>
-  </si>
-  <si>
-    <t>AttractionFishType</t>
-  </si>
-  <si>
-    <t>bait_basic</t>
-  </si>
-  <si>
-    <t>기본 미끼</t>
-  </si>
-  <si>
-    <t>all</t>
-  </si>
-  <si>
-    <t>아무 물고기나 잡을 수 있는 기본 미끼입니다.</t>
-  </si>
-  <si>
-    <t>bait_worm</t>
-  </si>
-  <si>
-    <t>지렁이</t>
-  </si>
-  <si>
-    <t>freshwater</t>
-  </si>
-  <si>
-    <t>민물고기에게 특히 효과적인 지렁이 미끼입니다.</t>
-  </si>
-  <si>
-    <t>bait_shrimp</t>
-  </si>
-  <si>
-    <t>새우</t>
-  </si>
-  <si>
-    <t>saltwater</t>
-  </si>
-  <si>
-    <t>바닷물고기에게 특히 효과적인 새우 미끼입니다.</t>
-  </si>
-  <si>
-    <t>bait_lure</t>
-  </si>
-  <si>
-    <t>루어</t>
-  </si>
-  <si>
-    <t>모든 물고기에게 효과가 좋은 인공 미끼입니다.</t>
-  </si>
-  <si>
-    <t>bait_golden</t>
-  </si>
-  <si>
-    <t>황금 미끼</t>
-  </si>
-  <si>
-    <t>rare</t>
-  </si>
-  <si>
-    <t>희귀 물고기를 유인하는 황금빛 미끼입니다.</t>
-  </si>
-  <si>
-    <t>bait_ancient</t>
-  </si>
-  <si>
-    <t>고대의 미끼</t>
-  </si>
-  <si>
-    <t>legendary</t>
-  </si>
-  <si>
-    <t>고대 바다 생물을 끌어당기는 신비로운 미끼입니다.</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="223">
+  <si>
+    <t xml:space="preserve">ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rank</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chance (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Price (Gold)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Min Length (cm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Max Length (cm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_alligator</t>
+  </si>
+  <si>
+    <t xml:space="preserve">악어</t>
+  </si>
+  <si>
+    <t xml:space="preserve">★★★★★</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_axolotl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">아홀로틀</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_bass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">큰입배스</t>
+  </si>
+  <si>
+    <t xml:space="preserve">★</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_bluegill</t>
+  </si>
+  <si>
+    <t xml:space="preserve">블루길</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_bowfin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">보우핀</t>
+  </si>
+  <si>
+    <t xml:space="preserve">★★</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_bullshark</t>
+  </si>
+  <si>
+    <t xml:space="preserve">황소상어</t>
+  </si>
+  <si>
+    <t xml:space="preserve">★★★★</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_carp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">잉어</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_catfish</t>
+  </si>
+  <si>
+    <t xml:space="preserve">메기</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_crab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">게</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_crappie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">크래피</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_crayfish</t>
+  </si>
+  <si>
+    <t xml:space="preserve">가재</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_drum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">민어</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_frog</t>
+  </si>
+  <si>
+    <t xml:space="preserve">개구리</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_gar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">가아</t>
+  </si>
+  <si>
+    <t xml:space="preserve">★★★</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_bass_golden</t>
+  </si>
+  <si>
+    <t xml:space="preserve">골든 배스</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_goldfish</t>
+  </si>
+  <si>
+    <t xml:space="preserve">금붕어</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_guppy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">구피</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_salmon_king</t>
+  </si>
+  <si>
+    <t xml:space="preserve">왕연어</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_koi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">비단잉어</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_leech</t>
+  </si>
+  <si>
+    <t xml:space="preserve">거머리</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_mooneye</t>
+  </si>
+  <si>
+    <t xml:space="preserve">문아이</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_muskellunge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">머스키</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_perch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">퍼치</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_pike</t>
+  </si>
+  <si>
+    <t xml:space="preserve">강꼬치고기</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_pupfish</t>
+  </si>
+  <si>
+    <t xml:space="preserve">펍피쉬</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_trout_rainbow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">무지개송어</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_salmon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">연어</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_snail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">달팽이</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_sturgeon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">철갑상어</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_toad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">두꺼비</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_turtle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">거북이</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_walleye</t>
+  </si>
+  <si>
+    <t xml:space="preserve">월아이</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_angelfish</t>
+  </si>
+  <si>
+    <t xml:space="preserve">엔젤피쉬</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_bluefish</t>
+  </si>
+  <si>
+    <t xml:space="preserve">블루피쉬</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_clownfish</t>
+  </si>
+  <si>
+    <t xml:space="preserve">흰동가리</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_coelacanth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">실러캔스</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_dogfish</t>
+  </si>
+  <si>
+    <t xml:space="preserve">돔발상어</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_eel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">장어</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_flounder</t>
+  </si>
+  <si>
+    <t xml:space="preserve">가자미</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_grouper</t>
+  </si>
+  <si>
+    <t xml:space="preserve">그루퍼</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_herring</t>
+  </si>
+  <si>
+    <t xml:space="preserve">청어</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_krill</t>
+  </si>
+  <si>
+    <t xml:space="preserve">크릴</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_lionfish</t>
+  </si>
+  <si>
+    <t xml:space="preserve">쏠배감펭</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_lobster</t>
+  </si>
+  <si>
+    <t xml:space="preserve">바닷가재</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_manowar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">만오워</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_mantaray</t>
+  </si>
+  <si>
+    <t xml:space="preserve">가오리</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_mantaray_golden</t>
+  </si>
+  <si>
+    <t xml:space="preserve">황금 가오리</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_seaturtle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">바다거북</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_anomalocaris</t>
+  </si>
+  <si>
+    <t xml:space="preserve">아노말로카리스</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_helicoprion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">헬리코프리온</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_leedsichthys</t>
+  </si>
+  <si>
+    <t xml:space="preserve">리드시크티스</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fish_ufo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UFO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EXP Reward</t>
+  </si>
+  <si>
+    <t xml:space="preserve">강의 지배자. 날카로운 이빨을 조심하세요.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">웃는 얼굴의 귀여운 도롱뇽. 보고만 있어도 기분이 좋아집니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">입이 정말 커서 무엇이든 집어삼키는 탐욕스러운 물고기입니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">평범하지만 특별한 당신만의 물고기입니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">바다의 최상위 포식자. 잡았다는 것 자체가 기적입니다!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">어항에서 탈출한 걸까요? 반짝이는 비늘이 아름답습니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">산호초 사이를 헤엄치는 귀여운 물고기. 영화 속 주인공 같아요.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">이건 물고기가 아닙니다! 외계에서 날아온 비행 물체네요.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weight</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Required Spam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Price</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CastDistanceBonus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CatchChanceBonus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Durability</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rod_basic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">기본 낚싯대</t>
+  </si>
+  <si>
+    <t xml:space="preserve">누구나 사용할 수 있는 기본 낚싯대입니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rod_carbon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">카본 낚싯대</t>
+  </si>
+  <si>
+    <t xml:space="preserve">가볍고 튼튼한 카본 소재의 낚싯대입니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rod_fiberglass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">유리섬유 낚싯대</t>
+  </si>
+  <si>
+    <t xml:space="preserve">유리섬유 소재로 제작된 중급 낚싯대입니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rod_titanium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">티타늄 낚싯대</t>
+  </si>
+  <si>
+    <t xml:space="preserve">초경량 티타늄 합금으로 제작된 고급 낚싯대입니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rod_legendary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">전설의 낚싯대</t>
+  </si>
+  <si>
+    <t xml:space="preserve">전설 속에만 존재한다는 궁극의 낚싯대입니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AttractionFishType</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bait_basic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">기본 미끼</t>
+  </si>
+  <si>
+    <t xml:space="preserve">all</t>
+  </si>
+  <si>
+    <t xml:space="preserve">아무 물고기나 잡을 수 있는 기본 미끼입니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bait_worm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">지렁이</t>
+  </si>
+  <si>
+    <t xml:space="preserve">freshwater</t>
+  </si>
+  <si>
+    <t xml:space="preserve">민물고기에게 특히 효과적인 지렁이 미끼입니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bait_shrimp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">새우</t>
+  </si>
+  <si>
+    <t xml:space="preserve">saltwater</t>
+  </si>
+  <si>
+    <t xml:space="preserve">바닷물고기에게 특히 효과적인 새우 미끼입니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bait_lure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">루어</t>
+  </si>
+  <si>
+    <t xml:space="preserve">모든 물고기에게 효과가 좋은 인공 미끼입니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bait_golden</t>
+  </si>
+  <si>
+    <t xml:space="preserve">황금 미끼</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rare</t>
+  </si>
+  <si>
+    <t xml:space="preserve">희귀 물고기를 유인하는 황금빛 미끼입니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bait_ancient</t>
+  </si>
+  <si>
+    <t xml:space="preserve">고대의 미끼</t>
+  </si>
+  <si>
+    <t xml:space="preserve">legendary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">고대 바다 생물을 끌어당기는 신비로운 미끼입니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">강의 지배자. 악어와 닮은 외모지만 물고기입니다. 날카로운 이빨을 조심하세요.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">영원히 어린 상태로 사는 귀여운 도롱뇽. 재생 능력이 놀랍습니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">입이 정말 커서 무엇이든 집어삼키는 탐욕스러운 민물 스타.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">파란 아가미 덮개가 매력적인 선버시. 아이들이 가장 좋아하는 물고기.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">공기 호흡이 가능한 원시 민물고기. 산소가 부족해도 끄떡없습니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">민물과 바닷물을 오르내리는 사나운 상어. 공격성이 매우 높습니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">민물의 거인. 튼튼하고 영리해서 낚시꾼의 단골 상대입니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">수염이 난 민물고기. 바닥을 더듬어 먹이를 찾습니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">옆으로 걷는 귀여운 갑각류. 집게발이지만 꽤 아픕니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">납작한 몸에 얼룩덜룩한 무늬. 낚시하기 재미있는 어종입니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">민물에 사는 작은 랍스터. 개울가 돌 밑에서 흔히 볼 수 있습니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">독특한 꽥꽥 소리를 내는 물고기. 북을 치는 것 같다고 해서 붙여진 이름.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">개구리? 아니요 물고기입니다. 물속과 육지를 넘나드는 양서류.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">악어처럼 긴 주둥이와 날카로운 이빨을 가진 민물의 공룡.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">황금빛으로 빛나는 특별한 배스. 행운을 부르는 물고기라고 합니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">어항에서 탈출한 금붕어. 반짝이는 비늘이 아름답습니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">형형색색의 꼬리를 가진 가장 작은 열대어 중 하나.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">왕연어. 연어 중에서도 가장 크고 힘이 셉니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">일본의 국민 물고기. 형형색색의 무늬가 마치 수중 그림입니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">빨판을 가진 기생 생물. 좀 징그럽지만 생태계의 중요한 구성원입니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">큰 눈이 달처럼 빛나는 야행성 물고기. 밤에 더 잘 잡힙니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">민물의 폭군. 북미 호수에서 최상위 포식자로 군림합니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">호수의 대표 어종. 초보 낚시꾼의 첫 번째 친구.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">민물 호수의 은밀한 사냥꾼. 수초 사이에 숨어있다가 기습합니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">사막의 물웅덩이에 사는 놀라운 생명체. 극한 환경에 적응했습니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">무지개처럼 화려한 색채의 송어. 깨끗한 물에서만 삽니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">태어난 강으로 돌아오는 신기한 물고기. 연어 회로도 유명하죠.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">천천히 그러나 꾸준히. 나선형 껍질이 아름다운 복족류입니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">철갑상어. 캐비어로 유명한 고대 어종, 비늘이 마치 갑옷 같습니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">울퉁불퉁한 피부가 매력 포인트. 독이 있으니 조심히 다루세요.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">등딱지를 지닌 느긋한 민물 거북. 수중 생활에 완벽히 적응했습니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">야간 투시경을 가진 민물고기. 어두운 물속에서도 먹이를 놓치지 않습니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">길게 늘어진 지느러미가 우아한 열대어. 수족관의 왕자님입니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">등푸른 생선의 대명사. 맛과 영양 모두 최고입니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주황색과 흰색 줄무늬가 사랑스러운 산호초의 아이돌.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">공룡 시대부터 살아남은 살아있는 화석. '바다의 공룡'이라 불립니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">작은 상어의 일종. 귀여운 외모와 달리 사냥 본능은 강합니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">뱀처럼 길고 미끈한 몸. 야행성이라 밤에 더 활발합니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">두 눈이 한쪽에 몰려 있는 납작 물고기. 해저 바닥에 완벽히 위장합니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">산호초의 잠복꾼. 바위 틈에 숨어있다가 한순간에 먹이를 덥썩.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">북해의 은빛 물결. 대량으로 떼지어 다니며 바다를 은빛으로 물들입니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">남극 바다의 작은 보석. 고래도 이 작은 생물을 먹고 삽니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">화려한 줄무늬와 독가시를 가진 위험한 미녀. 절대 만지면 안 됩니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">바다의 갑옷 기사. 큰 집게발로 먹이를 움켜잡습니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">바다의 독가스 풍선. 긴 촉수에 치명적인 독이 있습니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">거대한 가오리가 우아하게 바다를 나는 듯 헤엄칩니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">황금빛 가오리. 햇빛에 반사되어 눈부시게 아름답습니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">고대부터 바다를 누빈 장수 거북. 등껍질에는 작은 생물들이 살고 있습니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">수억 년 전 고대 바다의 포식자. 살아있는 화석이라 불리기에 손색없는 존재입니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">톱니처럼 말려 있는 이빨이 인상적인 고대 상어. 독특한 턱 구조를 가졌습니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">고대 바다의 거대 여과 섭식자. 몸집은 크지만 성격은 온순합니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">이건 물고기가 아닙니다! 외계에서 날아온 미확인 비행 물체. 반짝이는 금속성 비늘을 가졌습니다.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -590,11 +741,11 @@
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    <ext uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -811,6 +962,7 @@
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
+          <a:custDash/>
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
@@ -818,6 +970,7 @@
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
+          <a:custDash/>
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
@@ -825,6 +978,7 @@
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
+          <a:custDash/>
           <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
@@ -896,7 +1050,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:K53"/>
   <sheetFormatPr defaultColWidth="8.375" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -958,7 +1112,7 @@
         <v>350</v>
       </c>
       <c r="H2" t="s">
-        <v>118</v>
+        <v>171</v>
       </c>
       <c r="I2">
         <v>5000</v>
@@ -993,13 +1147,13 @@
         <v>25</v>
       </c>
       <c r="H3" t="s">
-        <v>119</v>
+        <v>172</v>
       </c>
       <c r="I3">
         <v>5000</v>
       </c>
       <c r="J3">
-        <v>3.0599999427795401</v>
+        <v>3.05999994277954</v>
       </c>
       <c r="K3">
         <v>7</v>
@@ -1028,13 +1182,13 @@
         <v>45</v>
       </c>
       <c r="H4" t="s">
-        <v>120</v>
+        <v>173</v>
       </c>
       <c r="I4">
         <v>20</v>
       </c>
       <c r="J4">
-        <v>2.1099998950958301</v>
+        <v>2.10999989509583</v>
       </c>
       <c r="K4">
         <v>3</v>
@@ -1063,13 +1217,13 @@
         <v>20</v>
       </c>
       <c r="H5" t="s">
-        <v>121</v>
+        <v>174</v>
       </c>
       <c r="I5">
         <v>20</v>
       </c>
       <c r="J5">
-        <v>0.44999998807907099</v>
+        <v>0.449999988079071</v>
       </c>
       <c r="K5">
         <v>2</v>
@@ -1098,7 +1252,7 @@
         <v>60</v>
       </c>
       <c r="H6" t="s">
-        <v>121</v>
+        <v>175</v>
       </c>
       <c r="I6">
         <v>80</v>
@@ -1133,7 +1287,7 @@
         <v>220</v>
       </c>
       <c r="H7" t="s">
-        <v>122</v>
+        <v>176</v>
       </c>
       <c r="I7">
         <v>1000</v>
@@ -1168,13 +1322,13 @@
         <v>70</v>
       </c>
       <c r="H8" t="s">
-        <v>121</v>
+        <v>177</v>
       </c>
       <c r="I8">
         <v>80</v>
       </c>
       <c r="J8">
-        <v>6.6599998474121103</v>
+        <v>6.65999984741211</v>
       </c>
       <c r="K8">
         <v>4</v>
@@ -1203,13 +1357,13 @@
         <v>80</v>
       </c>
       <c r="H9" t="s">
-        <v>121</v>
+        <v>178</v>
       </c>
       <c r="I9">
         <v>20</v>
       </c>
       <c r="J9">
-        <v>7.1999998092651403</v>
+        <v>7.19999980926514</v>
       </c>
       <c r="K9">
         <v>3</v>
@@ -1238,13 +1392,13 @@
         <v>15</v>
       </c>
       <c r="H10" t="s">
-        <v>121</v>
+        <v>179</v>
       </c>
       <c r="I10">
         <v>20</v>
       </c>
       <c r="J10">
-        <v>0.20000000298023199</v>
+        <v>0.200000002980232</v>
       </c>
       <c r="K10">
         <v>2</v>
@@ -1273,13 +1427,13 @@
         <v>25</v>
       </c>
       <c r="H11" t="s">
-        <v>121</v>
+        <v>180</v>
       </c>
       <c r="I11">
         <v>20</v>
       </c>
       <c r="J11">
-        <v>0.80000001192092896</v>
+        <v>0.800000011920929</v>
       </c>
       <c r="K11">
         <v>2</v>
@@ -1308,7 +1462,7 @@
         <v>10</v>
       </c>
       <c r="H12" t="s">
-        <v>121</v>
+        <v>181</v>
       </c>
       <c r="I12">
         <v>20</v>
@@ -1343,13 +1497,13 @@
         <v>50</v>
       </c>
       <c r="H13" t="s">
-        <v>121</v>
+        <v>182</v>
       </c>
       <c r="I13">
         <v>80</v>
       </c>
       <c r="J13">
-        <v>3.0899999141693102</v>
+        <v>3.08999991416931</v>
       </c>
       <c r="K13">
         <v>4</v>
@@ -1378,13 +1532,13 @@
         <v>8</v>
       </c>
       <c r="H14" t="s">
-        <v>121</v>
+        <v>183</v>
       </c>
       <c r="I14">
         <v>20</v>
       </c>
       <c r="J14">
-        <v>5.9999998658895499E-2</v>
+        <v>0.0599999986588955</v>
       </c>
       <c r="K14">
         <v>2</v>
@@ -1413,13 +1567,13 @@
         <v>150</v>
       </c>
       <c r="H15" t="s">
-        <v>121</v>
+        <v>184</v>
       </c>
       <c r="I15">
         <v>250</v>
       </c>
       <c r="J15">
-        <v>39.680000305175803</v>
+        <v>39.6800003051758</v>
       </c>
       <c r="K15">
         <v>6</v>
@@ -1448,7 +1602,7 @@
         <v>50</v>
       </c>
       <c r="H16" t="s">
-        <v>120</v>
+        <v>185</v>
       </c>
       <c r="I16">
         <v>5000</v>
@@ -1483,13 +1637,13 @@
         <v>15</v>
       </c>
       <c r="H17" t="s">
-        <v>123</v>
+        <v>186</v>
       </c>
       <c r="I17">
         <v>20</v>
       </c>
       <c r="J17">
-        <v>0.20000000298023199</v>
+        <v>0.200000002980232</v>
       </c>
       <c r="K17">
         <v>2</v>
@@ -1518,13 +1672,13 @@
         <v>5</v>
       </c>
       <c r="H18" t="s">
-        <v>121</v>
+        <v>187</v>
       </c>
       <c r="I18">
         <v>20</v>
       </c>
       <c r="J18">
-        <v>1.9999999552965199E-2</v>
+        <v>0.0199999995529652</v>
       </c>
       <c r="K18">
         <v>2</v>
@@ -1553,7 +1707,7 @@
         <v>120</v>
       </c>
       <c r="H19" t="s">
-        <v>121</v>
+        <v>188</v>
       </c>
       <c r="I19">
         <v>1000</v>
@@ -1588,13 +1742,13 @@
         <v>65</v>
       </c>
       <c r="H20" t="s">
-        <v>121</v>
+        <v>189</v>
       </c>
       <c r="I20">
         <v>250</v>
       </c>
       <c r="J20">
-        <v>6.7699999809265101</v>
+        <v>6.76999998092651</v>
       </c>
       <c r="K20">
         <v>5</v>
@@ -1623,13 +1777,13 @@
         <v>5</v>
       </c>
       <c r="H21" t="s">
-        <v>121</v>
+        <v>190</v>
       </c>
       <c r="I21">
         <v>20</v>
       </c>
       <c r="J21">
-        <v>1.9999999552965199E-2</v>
+        <v>0.0199999995529652</v>
       </c>
       <c r="K21">
         <v>2</v>
@@ -1658,13 +1812,13 @@
         <v>30</v>
       </c>
       <c r="H22" t="s">
-        <v>121</v>
+        <v>191</v>
       </c>
       <c r="I22">
         <v>80</v>
       </c>
       <c r="J22">
-        <v>1.1100000143051101</v>
+        <v>1.11000001430511</v>
       </c>
       <c r="K22">
         <v>3</v>
@@ -1693,7 +1847,7 @@
         <v>130</v>
       </c>
       <c r="H23" t="s">
-        <v>121</v>
+        <v>192</v>
       </c>
       <c r="I23">
         <v>250</v>
@@ -1728,7 +1882,7 @@
         <v>35</v>
       </c>
       <c r="H24" t="s">
-        <v>121</v>
+        <v>193</v>
       </c>
       <c r="I24">
         <v>20</v>
@@ -1763,13 +1917,13 @@
         <v>100</v>
       </c>
       <c r="H25" t="s">
-        <v>121</v>
+        <v>194</v>
       </c>
       <c r="I25">
         <v>250</v>
       </c>
       <c r="J25">
-        <v>16.879999160766602</v>
+        <v>16.8799991607666</v>
       </c>
       <c r="K25">
         <v>6</v>
@@ -1798,13 +1952,13 @@
         <v>4</v>
       </c>
       <c r="H26" t="s">
-        <v>121</v>
+        <v>195</v>
       </c>
       <c r="I26">
         <v>20</v>
       </c>
       <c r="J26">
-        <v>9.9999997764825804E-3</v>
+        <v>0.00999999977648258</v>
       </c>
       <c r="K26">
         <v>2</v>
@@ -1833,13 +1987,13 @@
         <v>55</v>
       </c>
       <c r="H27" t="s">
-        <v>121</v>
+        <v>196</v>
       </c>
       <c r="I27">
         <v>250</v>
       </c>
       <c r="J27">
-        <v>5.4200000762939498</v>
+        <v>5.42000007629395</v>
       </c>
       <c r="K27">
         <v>5</v>
@@ -1868,13 +2022,13 @@
         <v>80</v>
       </c>
       <c r="H28" t="s">
-        <v>121</v>
+        <v>197</v>
       </c>
       <c r="I28">
         <v>80</v>
       </c>
       <c r="J28">
-        <v>7.9200000762939498</v>
+        <v>7.92000007629395</v>
       </c>
       <c r="K28">
         <v>4</v>
@@ -1903,13 +2057,13 @@
         <v>3</v>
       </c>
       <c r="H29" t="s">
-        <v>121</v>
+        <v>198</v>
       </c>
       <c r="I29">
         <v>20</v>
       </c>
       <c r="J29">
-        <v>9.9999997764825804E-3</v>
+        <v>0.00999999977648258</v>
       </c>
       <c r="K29">
         <v>2</v>
@@ -1938,13 +2092,13 @@
         <v>250</v>
       </c>
       <c r="H30" t="s">
-        <v>121</v>
+        <v>199</v>
       </c>
       <c r="I30">
         <v>1000</v>
       </c>
       <c r="J30">
-        <v>153.11999511718801</v>
+        <v>153.119995117188</v>
       </c>
       <c r="K30">
         <v>8</v>
@@ -1973,7 +2127,7 @@
         <v>12</v>
       </c>
       <c r="H31" t="s">
-        <v>121</v>
+        <v>200</v>
       </c>
       <c r="I31">
         <v>20</v>
@@ -2008,7 +2162,7 @@
         <v>40</v>
       </c>
       <c r="H32" t="s">
-        <v>121</v>
+        <v>201</v>
       </c>
       <c r="I32">
         <v>80</v>
@@ -2043,13 +2197,13 @@
         <v>60</v>
       </c>
       <c r="H33" t="s">
-        <v>121</v>
+        <v>202</v>
       </c>
       <c r="I33">
         <v>250</v>
       </c>
       <c r="J33">
-        <v>6.0799999237060502</v>
+        <v>6.07999992370605</v>
       </c>
       <c r="K33">
         <v>5</v>
@@ -2078,7 +2232,7 @@
         <v>20</v>
       </c>
       <c r="H34" t="s">
-        <v>121</v>
+        <v>203</v>
       </c>
       <c r="I34">
         <v>1000</v>
@@ -2113,13 +2267,13 @@
         <v>50</v>
       </c>
       <c r="H35" t="s">
-        <v>121</v>
+        <v>204</v>
       </c>
       <c r="I35">
         <v>20</v>
       </c>
       <c r="J35">
-        <v>2.8099999427795401</v>
+        <v>2.80999994277954</v>
       </c>
       <c r="K35">
         <v>3</v>
@@ -2148,7 +2302,7 @@
         <v>10</v>
       </c>
       <c r="H36" t="s">
-        <v>124</v>
+        <v>205</v>
       </c>
       <c r="I36">
         <v>20</v>
@@ -2183,7 +2337,7 @@
         <v>180</v>
       </c>
       <c r="H37" t="s">
-        <v>121</v>
+        <v>206</v>
       </c>
       <c r="I37">
         <v>5000</v>
@@ -2218,7 +2372,7 @@
         <v>100</v>
       </c>
       <c r="H38" t="s">
-        <v>121</v>
+        <v>207</v>
       </c>
       <c r="I38">
         <v>80</v>
@@ -2253,13 +2407,13 @@
         <v>110</v>
       </c>
       <c r="H39" t="s">
-        <v>121</v>
+        <v>208</v>
       </c>
       <c r="I39">
         <v>20</v>
       </c>
       <c r="J39">
-        <v>14.449999809265099</v>
+        <v>14.4499998092651</v>
       </c>
       <c r="K39">
         <v>4</v>
@@ -2288,7 +2442,7 @@
         <v>40</v>
       </c>
       <c r="H40" t="s">
-        <v>121</v>
+        <v>209</v>
       </c>
       <c r="I40">
         <v>20</v>
@@ -2323,13 +2477,13 @@
         <v>150</v>
       </c>
       <c r="H41" t="s">
-        <v>121</v>
+        <v>210</v>
       </c>
       <c r="I41">
         <v>250</v>
       </c>
       <c r="J41">
-        <v>39.680000305175803</v>
+        <v>39.6800003051758</v>
       </c>
       <c r="K41">
         <v>6</v>
@@ -2358,13 +2512,13 @@
         <v>30</v>
       </c>
       <c r="H42" t="s">
-        <v>121</v>
+        <v>211</v>
       </c>
       <c r="I42">
         <v>20</v>
       </c>
       <c r="J42">
-        <v>1.0099999904632599</v>
+        <v>1.00999999046326</v>
       </c>
       <c r="K42">
         <v>2</v>
@@ -2393,7 +2547,7 @@
         <v>2</v>
       </c>
       <c r="H43" t="s">
-        <v>121</v>
+        <v>212</v>
       </c>
       <c r="I43">
         <v>20</v>
@@ -2428,7 +2582,7 @@
         <v>35</v>
       </c>
       <c r="H44" t="s">
-        <v>121</v>
+        <v>213</v>
       </c>
       <c r="I44">
         <v>250</v>
@@ -2463,13 +2617,13 @@
         <v>45</v>
       </c>
       <c r="H45" t="s">
-        <v>121</v>
+        <v>214</v>
       </c>
       <c r="I45">
         <v>1000</v>
       </c>
       <c r="J45">
-        <v>5.2800002098083496</v>
+        <v>5.28000020980835</v>
       </c>
       <c r="K45">
         <v>6</v>
@@ -2498,13 +2652,13 @@
         <v>30</v>
       </c>
       <c r="H46" t="s">
-        <v>121</v>
+        <v>215</v>
       </c>
       <c r="I46">
         <v>1000</v>
       </c>
       <c r="J46">
-        <v>2.5299999713897701</v>
+        <v>2.52999997138977</v>
       </c>
       <c r="K46">
         <v>6</v>
@@ -2533,13 +2687,13 @@
         <v>250</v>
       </c>
       <c r="H47" t="s">
-        <v>121</v>
+        <v>216</v>
       </c>
       <c r="I47">
         <v>250</v>
       </c>
       <c r="J47">
-        <v>91.879997253417997</v>
+        <v>91.879997253418</v>
       </c>
       <c r="K47">
         <v>7</v>
@@ -2568,7 +2722,7 @@
         <v>300</v>
       </c>
       <c r="H48" t="s">
-        <v>121</v>
+        <v>217</v>
       </c>
       <c r="I48">
         <v>5000</v>
@@ -2603,7 +2757,7 @@
         <v>120</v>
       </c>
       <c r="H49" t="s">
-        <v>121</v>
+        <v>218</v>
       </c>
       <c r="I49">
         <v>5000</v>
@@ -2638,7 +2792,7 @@
         <v>100</v>
       </c>
       <c r="H50" t="s">
-        <v>121</v>
+        <v>219</v>
       </c>
       <c r="I50">
         <v>5000</v>
@@ -2673,7 +2827,7 @@
         <v>400</v>
       </c>
       <c r="H51" t="s">
-        <v>121</v>
+        <v>220</v>
       </c>
       <c r="I51">
         <v>5000</v>
@@ -2708,7 +2862,7 @@
         <v>1600</v>
       </c>
       <c r="H52" t="s">
-        <v>121</v>
+        <v>221</v>
       </c>
       <c r="I52">
         <v>5000</v>
@@ -2743,7 +2897,7 @@
         <v>500</v>
       </c>
       <c r="H53" t="s">
-        <v>125</v>
+        <v>222</v>
       </c>
       <c r="I53">
         <v>5000</v>

</xml_diff>